<commit_message>
fix: atualizar observações padrão riscos 7/9/13, corrigir bug SEL_RISCOS e adicionar aba banco de riscos no Excel
- RISCO 7: adicionar distâncias mínimas 345 kV (3,5 m) e 138 kV (1,5 m) como obs. padrão
- RISCO 9: adicionar verificação de malha terra e equipotencialização como obs. padrão
- RISCO 13: remover 'Máscara contra UV para solda' da descrição
- Bug fix: restaurar SEL_RISCOS a partir de fase._riscos em renderRiscosSel() para preservar riscos de APRs persistidas após nova()
- Docs: corrigir contagem EQUIPE_CAMPO de 46 → 45 no comentário
- Excel: adicionar aba 'Banco de Riscos' com 35 riscos completos (R07, R09, R13 marcados em verde)
- Excel: atualizar data 'Última atualização' para 18/06/2026 na aba Visão Geral

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/APR_REMO_Historico_Projeto.xlsx
+++ b/APR_REMO_Historico_Projeto.xlsx
@@ -1,23 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Remo Engenharia\Desktop\apr\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{859A0F83-F694-4BA2-B279-61CD8451D50F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C376562-E6C1-4CF9-87BA-905C9768F8CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8196" yWindow="696" windowWidth="12492" windowHeight="10920" firstSheet="3" activeTab="4" xr2:uid="{E8D2854C-CAA7-4AC3-9D15-57F2C505D09B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="4" xr2:uid="{E8D2854C-CAA7-4AC3-9D15-57F2C505D09B}"/>
   </bookViews>
   <sheets>
     <sheet name="Visão Geral" sheetId="1" r:id="rId1"/>
     <sheet name="Histórico de Commits" sheetId="2" r:id="rId2"/>
     <sheet name="Funcionalidades" sheetId="3" r:id="rId3"/>
     <sheet name="Banco de Dados" sheetId="4" r:id="rId4"/>
-    <sheet name="Integração Drive" sheetId="5" r:id="rId5"/>
+    <sheet name="Banco de Riscos" sheetId="6" r:id="rId5"/>
+    <sheet name="Integração Drive" sheetId="5" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="278">
   <si>
     <t>SISTEMA APR DIGITAL — REMO ENGENHARIA</t>
   </si>
@@ -614,13 +615,271 @@
   </si>
   <si>
     <t>registrarPlanilha: appendRow 13 colunas + richText 'Abrir PDF' com hyperlink na coluna 7</t>
+  </si>
+  <si>
+    <t>BANCO DE RISCOS — SISTEMA APR REMO ENGENHARIA</t>
+  </si>
+  <si>
+    <t>SE JAGUARA 345 kV  |  35 Riscos com Probabilidade, Severidade e Medidas de Controle</t>
+  </si>
+  <si>
+    <t>Nº</t>
+  </si>
+  <si>
+    <t>Prob.</t>
+  </si>
+  <si>
+    <t>Sev.</t>
+  </si>
+  <si>
+    <t>Risco / Perigo</t>
+  </si>
+  <si>
+    <t>Medida de Controle Padrão</t>
+  </si>
+  <si>
+    <t>Média</t>
+  </si>
+  <si>
+    <t>Moderada</t>
+  </si>
+  <si>
+    <t>Cansaço Físico/Mental</t>
+  </si>
+  <si>
+    <t>Verificar condições físicas e psicológicas dos integrantes da equipe através do emociograma do DSS.</t>
+  </si>
+  <si>
+    <t>Grave</t>
+  </si>
+  <si>
+    <t>Uso de Adorno</t>
+  </si>
+  <si>
+    <t>É proibido executar atividades portando adornos (anéis, brincos, aliança, colar, celular).</t>
+  </si>
+  <si>
+    <t>Impacto Ambiental</t>
+  </si>
+  <si>
+    <t>Todos os resíduos gerados devem ser descartados corretamente. Área deve estar limpa e organizada.</t>
+  </si>
+  <si>
+    <t>Uso de Ferramentas Inadequadas</t>
+  </si>
+  <si>
+    <t>Não improvisar ferramentas. Realizar checklist antes do uso. Nunca utilizar ferramentas danificadas.</t>
+  </si>
+  <si>
+    <t>Procedimentos Técnicos Incorretos</t>
+  </si>
+  <si>
+    <t>Comunicação direta e simplificada. Direcionar função por colaborador. Recolher assinaturas ao término.</t>
+  </si>
+  <si>
+    <t>Picadas de Animais Peçonhentos</t>
+  </si>
+  <si>
+    <t>Verificar presença de animais peçonhentos antes de iniciar atividades em escavações.</t>
+  </si>
+  <si>
+    <t>Alta</t>
+  </si>
+  <si>
+    <t>Crítica</t>
+  </si>
+  <si>
+    <t>Trabalho próx. a Circuitos Energizados</t>
+  </si>
+  <si>
+    <t>Manter distâncias de segurança dos pontos energizados. 345 kV Distância mínima de aproximação: 3,5 metros - 138 kV Distância mínima de aproximação: 1,5 metros.</t>
+  </si>
+  <si>
+    <t>Retorno de Tensão</t>
+  </si>
+  <si>
+    <t>Certificar liberação do equipamento. Aterramento provisório. Teste de ausência de tensão. LOTO.</t>
+  </si>
+  <si>
+    <t>Indução Elétrica</t>
+  </si>
+  <si>
+    <t>Utilizar aterramento provisório. Inspecionar cabos de aterramento. Apresentar distâncias de segurança. Verificar se área contém malha terra eficiente para garantir a equipotencialização e uso de isolantes para evitar contato acidental com partes energizadas.</t>
+  </si>
+  <si>
+    <t>Trip Acidental</t>
+  </si>
+  <si>
+    <t>Seguir procedimento de bloqueio e etiquetagem conforme NR-10.</t>
+  </si>
+  <si>
+    <t>Choque Elétrico</t>
+  </si>
+  <si>
+    <t>Proibido materiais metálicos próx. a SEP. Inspecionar extensões/cabos. Proibido trenas metálicas.</t>
+  </si>
+  <si>
+    <t>Exposição a Ruído</t>
+  </si>
+  <si>
+    <t>Fazer uso de protetor auricular tipo plug ou concha.</t>
+  </si>
+  <si>
+    <t>Leve</t>
+  </si>
+  <si>
+    <t>Exposição à Radiação</t>
+  </si>
+  <si>
+    <t>Usar protetor solar e reaplicar a cada 2 horas. Manter hidratação.</t>
+  </si>
+  <si>
+    <t>Queda em Altura</t>
+  </si>
+  <si>
+    <t>Treinamento NR-35 obrigatório. Cinto paraquedista com dois talabartes acima de 2 m. PT necessária.</t>
+  </si>
+  <si>
+    <t>Exposição a Vibrações</t>
+  </si>
+  <si>
+    <t>Rodízio entre profissionais: 25 min trabalhados / 10 min descanso. Luva anti-vibração.</t>
+  </si>
+  <si>
+    <t>Exposição a Fumos Metálicos</t>
+  </si>
+  <si>
+    <t>Usar máscara de proteção adequada para fumos e ventilação no local.</t>
+  </si>
+  <si>
+    <t>Incêndio / Explosões</t>
+  </si>
+  <si>
+    <t>Manter extintor de incêndio próximo. Verificar ausência de materiais inflamáveis na área.</t>
+  </si>
+  <si>
+    <t>Exposição a Poeiras</t>
+  </si>
+  <si>
+    <t>Uso obrigatório de máscara PFF2 para proteção de poeira.</t>
+  </si>
+  <si>
+    <t>Levantamento Manual de Peso</t>
+  </si>
+  <si>
+    <t>Evitar levantar peso excessivo sozinho. Técnica correta: coluna ereta, força das pernas. Máx. 23 kg.</t>
+  </si>
+  <si>
+    <t>Prensamento de Membros</t>
+  </si>
+  <si>
+    <t>Manter o corpo fora do raio de ação do equipamento.</t>
+  </si>
+  <si>
+    <t>Colisões / Abalroamento</t>
+  </si>
+  <si>
+    <t>Transitar apenas nos locais destinados à tarefa. Delimitar área com cones, cordas e acessórios.</t>
+  </si>
+  <si>
+    <t>Baixa</t>
+  </si>
+  <si>
+    <t>Iluminação Inadequada</t>
+  </si>
+  <si>
+    <t>Garantir iluminação adequada no local de trabalho antes de iniciar atividades noturnas ou em ambientes fechados.</t>
+  </si>
+  <si>
+    <t>Exposição a Gases/Vapores</t>
+  </si>
+  <si>
+    <t>Armazenar combustível somente em local autorizado. Extintor de incêndio no local dentro do prazo.</t>
+  </si>
+  <si>
+    <t>Atropelamento</t>
+  </si>
+  <si>
+    <t>Atentar ao trajeto perante veículos e máquinas. Contato visual com motorista e sinaleiro.</t>
+  </si>
+  <si>
+    <t>Máquinas sem Proteção</t>
+  </si>
+  <si>
+    <t>Verificar proteções de máquinas conforme NR-12 antes de operar. Nunca remover proteções.</t>
+  </si>
+  <si>
+    <t>Contato com Produtos Químicos</t>
+  </si>
+  <si>
+    <t>Uso obrigatório de luvas nitrílicas e máscara PFF2. Consultar FISPQ dos produtos manuseados.</t>
+  </si>
+  <si>
+    <t>Manobra ou Operação Indevida</t>
+  </si>
+  <si>
+    <t>Operação somente por profissionais autorizados. Rádio de comunicação. Área sinalizada e isolada.</t>
+  </si>
+  <si>
+    <t>Escoriações / Cortes / Pancadas</t>
+  </si>
+  <si>
+    <t>Utilizar luvas de vaqueta. Delimitar área de trabalho com cones e cordas.</t>
+  </si>
+  <si>
+    <t>Projeção de Partículas</t>
+  </si>
+  <si>
+    <t>Uso obrigatório de óculos de proteção durante todo o processo.</t>
+  </si>
+  <si>
+    <t>Falha / Falta de Comunicação</t>
+  </si>
+  <si>
+    <t>Repassar perigos e controles. Comunicação clara e objetiva. Sanar dúvidas antes de iniciar.</t>
+  </si>
+  <si>
+    <t>Condições Meteorológicas Adversas</t>
+  </si>
+  <si>
+    <t>Suspender atividades em caso de raios e trovadas. Seguir fluxo de comunicação de acidentes (PAE).</t>
+  </si>
+  <si>
+    <t>Desmoronamento / Soterramento</t>
+  </si>
+  <si>
+    <t>Avaliar condições do solo. Proibir permanência na base do talude sem proteção. Sinalizar e isolar área de risco.</t>
+  </si>
+  <si>
+    <t>Queda de Materiais e Ferramentas</t>
+  </si>
+  <si>
+    <t>Manter ferramentas próximas ao local de trabalho. Área limpa e organizada continuamente.</t>
+  </si>
+  <si>
+    <t>Queda de Pessoas</t>
+  </si>
+  <si>
+    <t>Executar limpeza contínua. Não acumular entulho em circulação. Comunicar áreas já limpas.</t>
+  </si>
+  <si>
+    <t>Queimaduras</t>
+  </si>
+  <si>
+    <t>Não se aproximar de partes quentes com a máquina ligada. Luvas de vaqueta e avental para solda.</t>
+  </si>
+  <si>
+    <t>* Riscos 07, 09 e 13 atualizados em 18/06/2026 — Observações padrão incluídas / Máscara UV removida do R13.</t>
+  </si>
+  <si>
+    <t>18/06/2026</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -716,8 +975,47 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF007A00"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -769,6 +1067,30 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF5F2ED"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00A651"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFBF9F7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEEFFDD"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE6F9FF"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -824,23 +1146,179 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -851,139 +1329,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1304,235 +1662,230 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{314DD115-A57B-4FE2-BE3B-EF13EE449DB6}">
   <dimension ref="A1:C26"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="28.77734375" customWidth="1"/>
-    <col min="2" max="2" width="54.77734375" customWidth="1"/>
-    <col min="3" max="3" width="20.77734375" customWidth="1"/>
+    <col min="1" max="1" width="28.7109375" customWidth="1"/>
+    <col min="2" max="2" width="54.7109375" customWidth="1"/>
+    <col min="3" max="3" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:3" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="57" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-    </row>
-    <row r="2" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="57"/>
+      <c r="C1" s="57"/>
+    </row>
+    <row r="2" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="58" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-    </row>
-    <row r="3" spans="1:3" ht="7.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-    </row>
-    <row r="4" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
+      <c r="B2" s="58"/>
+      <c r="C2" s="58"/>
+    </row>
+    <row r="3" spans="1:3" ht="7.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+    </row>
+    <row r="4" spans="1:3" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="55" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="5"/>
-    </row>
-    <row r="5" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
+      <c r="C4" s="56"/>
+    </row>
+    <row r="5" spans="1:3" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="55" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="5"/>
-    </row>
-    <row r="6" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
+      <c r="C5" s="56"/>
+    </row>
+    <row r="6" spans="1:3" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="55" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="5"/>
-    </row>
-    <row r="7" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
+      <c r="C6" s="56"/>
+    </row>
+    <row r="7" spans="1:3" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="55" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="5"/>
-    </row>
-    <row r="8" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
+      <c r="C7" s="56"/>
+    </row>
+    <row r="8" spans="1:3" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="55" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="5"/>
-    </row>
-    <row r="9" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
+      <c r="C8" s="56"/>
+    </row>
+    <row r="9" spans="1:3" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="55" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="5"/>
-    </row>
-    <row r="10" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
+      <c r="C9" s="56"/>
+    </row>
+    <row r="10" spans="1:3" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="6">
+      <c r="B10" s="55">
         <v>4.0999999999999996</v>
       </c>
-      <c r="C10" s="5"/>
-    </row>
-    <row r="11" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="4" t="s">
+      <c r="C10" s="56"/>
+    </row>
+    <row r="11" spans="1:3" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="55" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="5"/>
-    </row>
-    <row r="12" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="4" t="s">
+      <c r="C11" s="56"/>
+    </row>
+    <row r="12" spans="1:3" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C12" s="5"/>
-    </row>
-    <row r="13" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="4" t="s">
+      <c r="B12" s="55" t="s">
+        <v>277</v>
+      </c>
+      <c r="C12" s="56"/>
+    </row>
+    <row r="13" spans="1:3" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="55" t="s">
         <v>20</v>
       </c>
-      <c r="C13" s="5"/>
-    </row>
-    <row r="14" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="4" t="s">
+      <c r="C13" s="56"/>
+    </row>
+    <row r="14" spans="1:3" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="55" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="5"/>
-    </row>
-    <row r="16" spans="1:3" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="7" t="s">
+      <c r="C14" s="56"/>
+    </row>
+    <row r="16" spans="1:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="61" t="s">
         <v>23</v>
       </c>
-      <c r="B16" s="7"/>
-      <c r="C16" s="7"/>
-    </row>
-    <row r="17" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="8" t="s">
+      <c r="B16" s="61"/>
+      <c r="C16" s="61"/>
+    </row>
+    <row r="17" spans="1:3" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="62" t="s">
         <v>25</v>
       </c>
-      <c r="C17" s="9"/>
-    </row>
-    <row r="18" spans="1:3" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="11" t="s">
+      <c r="C17" s="63"/>
+    </row>
+    <row r="18" spans="1:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B18" s="13" t="s">
+      <c r="B18" s="59" t="s">
         <v>27</v>
       </c>
-      <c r="C18" s="12"/>
-    </row>
-    <row r="19" spans="1:3" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="14" t="s">
+      <c r="C18" s="60"/>
+    </row>
+    <row r="19" spans="1:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="15" t="s">
+      <c r="B19" s="64" t="s">
         <v>29</v>
       </c>
-      <c r="C19" s="12"/>
-    </row>
-    <row r="20" spans="1:3" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="11" t="s">
+      <c r="C19" s="60"/>
+    </row>
+    <row r="20" spans="1:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B20" s="13" t="s">
+      <c r="B20" s="59" t="s">
         <v>31</v>
       </c>
-      <c r="C20" s="12"/>
-    </row>
-    <row r="21" spans="1:3" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="14" t="s">
+      <c r="C20" s="60"/>
+    </row>
+    <row r="21" spans="1:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B21" s="15" t="s">
+      <c r="B21" s="64" t="s">
         <v>33</v>
       </c>
-      <c r="C21" s="12"/>
-    </row>
-    <row r="22" spans="1:3" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="11" t="s">
+      <c r="C21" s="60"/>
+    </row>
+    <row r="22" spans="1:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="B22" s="13" t="s">
+      <c r="B22" s="59" t="s">
         <v>35</v>
       </c>
-      <c r="C22" s="12"/>
-    </row>
-    <row r="23" spans="1:3" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="14" t="s">
+      <c r="C22" s="60"/>
+    </row>
+    <row r="23" spans="1:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B23" s="15" t="s">
+      <c r="B23" s="64" t="s">
         <v>37</v>
       </c>
-      <c r="C23" s="12"/>
-    </row>
-    <row r="24" spans="1:3" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="11" t="s">
+      <c r="C23" s="60"/>
+    </row>
+    <row r="24" spans="1:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B24" s="13" t="s">
+      <c r="B24" s="59" t="s">
         <v>39</v>
       </c>
-      <c r="C24" s="12"/>
-    </row>
-    <row r="25" spans="1:3" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="14" t="s">
+      <c r="C24" s="60"/>
+    </row>
+    <row r="25" spans="1:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="B25" s="15" t="s">
+      <c r="B25" s="64" t="s">
         <v>41</v>
       </c>
-      <c r="C25" s="12"/>
-    </row>
-    <row r="26" spans="1:3" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="11" t="s">
+      <c r="C25" s="60"/>
+    </row>
+    <row r="26" spans="1:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B26" s="13" t="s">
+      <c r="B26" s="59" t="s">
         <v>43</v>
       </c>
-      <c r="C26" s="12"/>
+      <c r="C26" s="60"/>
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B25:C25"/>
     <mergeCell ref="B26:C26"/>
     <mergeCell ref="B14:C14"/>
     <mergeCell ref="A16:C16"/>
@@ -1540,11 +1893,11 @@
     <mergeCell ref="B18:C18"/>
     <mergeCell ref="B19:C19"/>
     <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:C2"/>
@@ -1552,6 +1905,11 @@
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
@@ -1560,179 +1918,179 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8EE7C958-1583-4AC7-AE30-B3B76C482C0D}">
   <dimension ref="A1:D13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.77734375" customWidth="1"/>
-    <col min="2" max="2" width="18.77734375" customWidth="1"/>
-    <col min="3" max="3" width="60.77734375" customWidth="1"/>
-    <col min="4" max="4" width="15.77734375" customWidth="1"/>
+    <col min="1" max="1" width="13.7109375" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" customWidth="1"/>
+    <col min="3" max="3" width="60.7109375" customWidth="1"/>
+    <col min="4" max="4" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="16" t="s">
+    <row r="1" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="65" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-    </row>
-    <row r="2" spans="1:4" ht="7.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-    </row>
-    <row r="3" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="8" t="s">
+      <c r="B1" s="65"/>
+      <c r="C1" s="65"/>
+      <c r="D1" s="65"/>
+    </row>
+    <row r="2" spans="1:4" ht="7.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+    </row>
+    <row r="3" spans="1:4" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="3" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="17" t="s">
+    <row r="4" spans="1:4" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="D4" s="20" t="s">
+      <c r="D4" s="11" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="17" t="s">
+    <row r="5" spans="1:4" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="D5" s="11" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="21" t="s">
+    <row r="6" spans="1:4" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="B6" s="22" t="s">
+      <c r="B6" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="C6" s="23" t="s">
+      <c r="C6" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="D6" s="24" t="s">
+      <c r="D6" s="15" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="21" t="s">
+    <row r="7" spans="1:4" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="B7" s="22" t="s">
+      <c r="B7" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="C7" s="23" t="s">
+      <c r="C7" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="D7" s="24" t="s">
+      <c r="D7" s="15" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="25" t="s">
+    <row r="8" spans="1:4" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="B8" s="26" t="s">
+      <c r="B8" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="C8" s="27" t="s">
+      <c r="C8" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="D8" s="28" t="s">
+      <c r="D8" s="19" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="25" t="s">
+    <row r="9" spans="1:4" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="B9" s="26" t="s">
+      <c r="B9" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="C9" s="27" t="s">
+      <c r="C9" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="D9" s="28" t="s">
+      <c r="D9" s="19" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="29" t="s">
+    <row r="10" spans="1:4" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="B10" s="30" t="s">
+      <c r="B10" s="21" t="s">
         <v>67</v>
       </c>
-      <c r="C10" s="31" t="s">
+      <c r="C10" s="22" t="s">
         <v>68</v>
       </c>
-      <c r="D10" s="32" t="s">
+      <c r="D10" s="23" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="33">
+    <row r="11" spans="1:4" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="24">
         <v>46178</v>
       </c>
-      <c r="B11" s="34" t="s">
+      <c r="B11" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="C11" s="35" t="s">
+      <c r="C11" s="26" t="s">
         <v>71</v>
       </c>
-      <c r="D11" s="36" t="s">
+      <c r="D11" s="27" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="37" t="s">
+    <row r="12" spans="1:4" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="28" t="s">
         <v>73</v>
       </c>
-      <c r="B12" s="38" t="s">
+      <c r="B12" s="29" t="s">
         <v>74</v>
       </c>
-      <c r="C12" s="39" t="s">
+      <c r="C12" s="30" t="s">
         <v>75</v>
       </c>
-      <c r="D12" s="40" t="s">
+      <c r="D12" s="31" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="41" t="s">
+    <row r="13" spans="1:4" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="42" t="s">
+      <c r="B13" s="33" t="s">
         <v>77</v>
       </c>
-      <c r="C13" s="43" t="s">
+      <c r="C13" s="34" t="s">
         <v>78</v>
       </c>
-      <c r="D13" s="44" t="s">
+      <c r="D13" s="35" t="s">
         <v>79</v>
       </c>
     </row>
@@ -1747,220 +2105,220 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{737883F1-38E5-492A-94D1-0A806479140D}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="28.77734375" customWidth="1"/>
-    <col min="2" max="2" width="54.77734375" customWidth="1"/>
-    <col min="3" max="3" width="14.77734375" customWidth="1"/>
+    <col min="1" max="1" width="28.7109375" customWidth="1"/>
+    <col min="2" max="2" width="54.7109375" customWidth="1"/>
+    <col min="3" max="3" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="16" t="s">
+    <row r="1" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="65" t="s">
         <v>80</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-    </row>
-    <row r="2" spans="1:3" ht="7.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-    </row>
-    <row r="3" spans="1:3" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="8" t="s">
+      <c r="B1" s="65"/>
+      <c r="C1" s="65"/>
+    </row>
+    <row r="2" spans="1:3" ht="7.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+    </row>
+    <row r="3" spans="1:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="3" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="11" t="s">
+    <row r="4" spans="1:3" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="B4" s="45" t="s">
+      <c r="B4" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="C4" s="46" t="s">
+      <c r="C4" s="36" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="14" t="s">
+    <row r="5" spans="1:3" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="B5" s="47" t="s">
+      <c r="B5" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="C5" s="48" t="s">
+      <c r="C5" s="37" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="11" t="s">
+    <row r="6" spans="1:3" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="B6" s="45" t="s">
+      <c r="B6" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="C6" s="46" t="s">
+      <c r="C6" s="36" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="14" t="s">
+    <row r="7" spans="1:3" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="B7" s="47" t="s">
+      <c r="B7" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="C7" s="48" t="s">
+      <c r="C7" s="37" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="11" t="s">
+    <row r="8" spans="1:3" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="B8" s="45" t="s">
+      <c r="B8" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="C8" s="46" t="s">
+      <c r="C8" s="36" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="14" t="s">
+    <row r="9" spans="1:3" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B9" s="47" t="s">
+      <c r="B9" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="C9" s="48" t="s">
+      <c r="C9" s="37" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="11" t="s">
+    <row r="10" spans="1:3" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="B10" s="45" t="s">
+      <c r="B10" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="C10" s="46" t="s">
+      <c r="C10" s="36" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="14" t="s">
+    <row r="11" spans="1:3" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="B11" s="47" t="s">
+      <c r="B11" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="C11" s="48" t="s">
+      <c r="C11" s="37" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="11" t="s">
+    <row r="12" spans="1:3" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="B12" s="45" t="s">
+      <c r="B12" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="C12" s="46" t="s">
+      <c r="C12" s="36" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="14" t="s">
+    <row r="13" spans="1:3" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="B13" s="47" t="s">
+      <c r="B13" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="C13" s="48" t="s">
+      <c r="C13" s="37" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="11" t="s">
+    <row r="14" spans="1:3" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="B14" s="45" t="s">
+      <c r="B14" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="C14" s="46" t="s">
+      <c r="C14" s="36" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="14" t="s">
+    <row r="15" spans="1:3" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="B15" s="47" t="s">
+      <c r="B15" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="C15" s="48" t="s">
+      <c r="C15" s="37" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="11" t="s">
+    <row r="16" spans="1:3" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="B16" s="45" t="s">
+      <c r="B16" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="C16" s="46" t="s">
+      <c r="C16" s="36" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="14" t="s">
+    <row r="17" spans="1:3" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="B17" s="47" t="s">
+      <c r="B17" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="C17" s="48" t="s">
+      <c r="C17" s="37" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="11" t="s">
+    <row r="18" spans="1:3" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="B18" s="45" t="s">
+      <c r="B18" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="C18" s="46" t="s">
+      <c r="C18" s="36" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="14" t="s">
+    <row r="19" spans="1:3" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="B19" s="47" t="s">
+      <c r="B19" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="C19" s="48" t="s">
+      <c r="C19" s="37" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="11" t="s">
+    <row r="20" spans="1:3" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="B20" s="45" t="s">
+      <c r="B20" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="C20" s="46" t="s">
+      <c r="C20" s="36" t="s">
         <v>86</v>
       </c>
     </row>
@@ -1975,175 +2333,175 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{804B6E00-6754-42FC-8EB8-A1D61B3F95A3}">
   <dimension ref="A1:D14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.77734375" customWidth="1"/>
-    <col min="2" max="2" width="11.77734375" customWidth="1"/>
-    <col min="3" max="3" width="46.77734375" customWidth="1"/>
-    <col min="4" max="4" width="22.77734375" customWidth="1"/>
+    <col min="1" max="1" width="22.7109375" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" customWidth="1"/>
+    <col min="3" max="3" width="46.7109375" customWidth="1"/>
+    <col min="4" max="4" width="22.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="16" t="s">
+    <row r="1" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="65" t="s">
         <v>119</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-    </row>
-    <row r="2" spans="1:4" ht="7.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-    </row>
-    <row r="3" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="8" t="s">
+      <c r="B1" s="65"/>
+      <c r="C1" s="65"/>
+      <c r="D1" s="65"/>
+    </row>
+    <row r="2" spans="1:4" ht="7.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+    </row>
+    <row r="3" spans="1:4" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="3" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="11" t="s">
+    <row r="4" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="B4" s="49">
+      <c r="B4" s="38">
         <v>32</v>
       </c>
-      <c r="C4" s="50" t="s">
+      <c r="C4" s="39" t="s">
         <v>124</v>
       </c>
-      <c r="D4" s="50" t="s">
+      <c r="D4" s="39" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="14" t="s">
+    <row r="5" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="B5" s="51">
+      <c r="B5" s="40">
         <v>35</v>
       </c>
-      <c r="C5" s="35" t="s">
+      <c r="C5" s="26" t="s">
         <v>127</v>
       </c>
-      <c r="D5" s="35" t="s">
+      <c r="D5" s="26" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="11" t="s">
+    <row r="6" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="B6" s="49">
+      <c r="B6" s="38">
         <v>46</v>
       </c>
-      <c r="C6" s="50" t="s">
+      <c r="C6" s="39" t="s">
         <v>130</v>
       </c>
-      <c r="D6" s="50" t="s">
+      <c r="D6" s="39" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="14" t="s">
+    <row r="7" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="B7" s="51">
+      <c r="B7" s="40">
         <v>7</v>
       </c>
-      <c r="C7" s="35" t="s">
+      <c r="C7" s="26" t="s">
         <v>133</v>
       </c>
-      <c r="D7" s="35" t="s">
+      <c r="D7" s="26" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="11" t="s">
+    <row r="8" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="B8" s="49" t="s">
+      <c r="B8" s="38" t="s">
         <v>136</v>
       </c>
-      <c r="C8" s="50" t="s">
+      <c r="C8" s="39" t="s">
         <v>137</v>
       </c>
-      <c r="D8" s="50" t="s">
+      <c r="D8" s="39" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="14" t="s">
+    <row r="9" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="B9" s="51">
+      <c r="B9" s="40">
         <v>33</v>
       </c>
-      <c r="C9" s="35" t="s">
+      <c r="C9" s="26" t="s">
         <v>140</v>
       </c>
-      <c r="D9" s="35" t="s">
+      <c r="D9" s="26" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="11" t="s">
+    <row r="10" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="B10" s="49">
+      <c r="B10" s="38">
         <v>14</v>
       </c>
-      <c r="C10" s="50" t="s">
+      <c r="C10" s="39" t="s">
         <v>143</v>
       </c>
-      <c r="D10" s="50" t="s">
+      <c r="D10" s="39" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="14" t="s">
+    <row r="11" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="B11" s="51">
+      <c r="B11" s="40">
         <v>28</v>
       </c>
-      <c r="C11" s="35" t="s">
+      <c r="C11" s="26" t="s">
         <v>146</v>
       </c>
-      <c r="D11" s="35" t="s">
+      <c r="D11" s="26" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="11" t="s">
+    <row r="12" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="B12" s="49">
+      <c r="B12" s="38">
         <v>2</v>
       </c>
-      <c r="C12" s="50" t="s">
+      <c r="C12" s="39" t="s">
         <v>148</v>
       </c>
-      <c r="D12" s="50" t="s">
+      <c r="D12" s="39" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="52" t="s">
+    <row r="14" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="66" t="s">
         <v>150</v>
       </c>
-      <c r="B14" s="52"/>
-      <c r="C14" s="52"/>
-      <c r="D14" s="52"/>
+      <c r="B14" s="66"/>
+      <c r="C14" s="66"/>
+      <c r="D14" s="66"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2155,213 +2513,875 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E05269C3-2D48-4CCF-8C6B-F49E7BE68237}">
+  <dimension ref="A1:E41"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="5.7109375" customWidth="1"/>
+    <col min="2" max="2" width="10.7109375" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" customWidth="1"/>
+    <col min="4" max="4" width="35.7109375" customWidth="1"/>
+    <col min="5" max="5" width="75.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="51" t="s">
+        <v>192</v>
+      </c>
+      <c r="B1" s="51"/>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="51"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="52" t="s">
+        <v>193</v>
+      </c>
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+    </row>
+    <row r="3" spans="1:5" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="41" t="s">
+        <v>194</v>
+      </c>
+      <c r="B4" s="41" t="s">
+        <v>195</v>
+      </c>
+      <c r="C4" s="41" t="s">
+        <v>196</v>
+      </c>
+      <c r="D4" s="41" t="s">
+        <v>197</v>
+      </c>
+      <c r="E4" s="41" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="43">
+        <v>1</v>
+      </c>
+      <c r="B5" s="44" t="s">
+        <v>199</v>
+      </c>
+      <c r="C5" s="44" t="s">
+        <v>200</v>
+      </c>
+      <c r="D5" s="42" t="s">
+        <v>201</v>
+      </c>
+      <c r="E5" s="42" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="46">
+        <v>2</v>
+      </c>
+      <c r="B6" s="47" t="s">
+        <v>199</v>
+      </c>
+      <c r="C6" s="47" t="s">
+        <v>203</v>
+      </c>
+      <c r="D6" s="45" t="s">
+        <v>204</v>
+      </c>
+      <c r="E6" s="45" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="43">
+        <v>3</v>
+      </c>
+      <c r="B7" s="44" t="s">
+        <v>199</v>
+      </c>
+      <c r="C7" s="44" t="s">
+        <v>200</v>
+      </c>
+      <c r="D7" s="42" t="s">
+        <v>206</v>
+      </c>
+      <c r="E7" s="42" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="46">
+        <v>4</v>
+      </c>
+      <c r="B8" s="47" t="s">
+        <v>199</v>
+      </c>
+      <c r="C8" s="47" t="s">
+        <v>200</v>
+      </c>
+      <c r="D8" s="45" t="s">
+        <v>208</v>
+      </c>
+      <c r="E8" s="45" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="43">
+        <v>5</v>
+      </c>
+      <c r="B9" s="44" t="s">
+        <v>199</v>
+      </c>
+      <c r="C9" s="44" t="s">
+        <v>203</v>
+      </c>
+      <c r="D9" s="42" t="s">
+        <v>210</v>
+      </c>
+      <c r="E9" s="42" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="46">
+        <v>6</v>
+      </c>
+      <c r="B10" s="47" t="s">
+        <v>199</v>
+      </c>
+      <c r="C10" s="47" t="s">
+        <v>200</v>
+      </c>
+      <c r="D10" s="45" t="s">
+        <v>212</v>
+      </c>
+      <c r="E10" s="45" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="50">
+        <v>7</v>
+      </c>
+      <c r="B11" s="49" t="s">
+        <v>214</v>
+      </c>
+      <c r="C11" s="49" t="s">
+        <v>215</v>
+      </c>
+      <c r="D11" s="48" t="s">
+        <v>216</v>
+      </c>
+      <c r="E11" s="48" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="46">
+        <v>8</v>
+      </c>
+      <c r="B12" s="47" t="s">
+        <v>199</v>
+      </c>
+      <c r="C12" s="47" t="s">
+        <v>215</v>
+      </c>
+      <c r="D12" s="45" t="s">
+        <v>218</v>
+      </c>
+      <c r="E12" s="45" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A13" s="50">
+        <v>9</v>
+      </c>
+      <c r="B13" s="49" t="s">
+        <v>214</v>
+      </c>
+      <c r="C13" s="49" t="s">
+        <v>203</v>
+      </c>
+      <c r="D13" s="48" t="s">
+        <v>220</v>
+      </c>
+      <c r="E13" s="48" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="46">
+        <v>10</v>
+      </c>
+      <c r="B14" s="47" t="s">
+        <v>199</v>
+      </c>
+      <c r="C14" s="47" t="s">
+        <v>203</v>
+      </c>
+      <c r="D14" s="45" t="s">
+        <v>222</v>
+      </c>
+      <c r="E14" s="45" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A15" s="43">
+        <v>11</v>
+      </c>
+      <c r="B15" s="44" t="s">
+        <v>199</v>
+      </c>
+      <c r="C15" s="44" t="s">
+        <v>215</v>
+      </c>
+      <c r="D15" s="42" t="s">
+        <v>224</v>
+      </c>
+      <c r="E15" s="42" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="46">
+        <v>12</v>
+      </c>
+      <c r="B16" s="47" t="s">
+        <v>214</v>
+      </c>
+      <c r="C16" s="47" t="s">
+        <v>200</v>
+      </c>
+      <c r="D16" s="45" t="s">
+        <v>226</v>
+      </c>
+      <c r="E16" s="45" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="50">
+        <v>13</v>
+      </c>
+      <c r="B17" s="49" t="s">
+        <v>214</v>
+      </c>
+      <c r="C17" s="49" t="s">
+        <v>228</v>
+      </c>
+      <c r="D17" s="48" t="s">
+        <v>229</v>
+      </c>
+      <c r="E17" s="48" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="46">
+        <v>14</v>
+      </c>
+      <c r="B18" s="47" t="s">
+        <v>199</v>
+      </c>
+      <c r="C18" s="47" t="s">
+        <v>215</v>
+      </c>
+      <c r="D18" s="45" t="s">
+        <v>231</v>
+      </c>
+      <c r="E18" s="45" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A19" s="43">
+        <v>15</v>
+      </c>
+      <c r="B19" s="44" t="s">
+        <v>199</v>
+      </c>
+      <c r="C19" s="44" t="s">
+        <v>200</v>
+      </c>
+      <c r="D19" s="42" t="s">
+        <v>233</v>
+      </c>
+      <c r="E19" s="42" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="46">
+        <v>16</v>
+      </c>
+      <c r="B20" s="47" t="s">
+        <v>199</v>
+      </c>
+      <c r="C20" s="47" t="s">
+        <v>200</v>
+      </c>
+      <c r="D20" s="45" t="s">
+        <v>235</v>
+      </c>
+      <c r="E20" s="45" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="43">
+        <v>17</v>
+      </c>
+      <c r="B21" s="44" t="s">
+        <v>199</v>
+      </c>
+      <c r="C21" s="44" t="s">
+        <v>215</v>
+      </c>
+      <c r="D21" s="42" t="s">
+        <v>237</v>
+      </c>
+      <c r="E21" s="42" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="46">
+        <v>18</v>
+      </c>
+      <c r="B22" s="47" t="s">
+        <v>214</v>
+      </c>
+      <c r="C22" s="47" t="s">
+        <v>228</v>
+      </c>
+      <c r="D22" s="45" t="s">
+        <v>239</v>
+      </c>
+      <c r="E22" s="45" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="43">
+        <v>19</v>
+      </c>
+      <c r="B23" s="44" t="s">
+        <v>214</v>
+      </c>
+      <c r="C23" s="44" t="s">
+        <v>200</v>
+      </c>
+      <c r="D23" s="42" t="s">
+        <v>241</v>
+      </c>
+      <c r="E23" s="42" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="46">
+        <v>20</v>
+      </c>
+      <c r="B24" s="47" t="s">
+        <v>199</v>
+      </c>
+      <c r="C24" s="47" t="s">
+        <v>203</v>
+      </c>
+      <c r="D24" s="45" t="s">
+        <v>243</v>
+      </c>
+      <c r="E24" s="45" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A25" s="43">
+        <v>21</v>
+      </c>
+      <c r="B25" s="44" t="s">
+        <v>199</v>
+      </c>
+      <c r="C25" s="44" t="s">
+        <v>203</v>
+      </c>
+      <c r="D25" s="42" t="s">
+        <v>245</v>
+      </c>
+      <c r="E25" s="42" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A26" s="46">
+        <v>22</v>
+      </c>
+      <c r="B26" s="47" t="s">
+        <v>247</v>
+      </c>
+      <c r="C26" s="47" t="s">
+        <v>200</v>
+      </c>
+      <c r="D26" s="45" t="s">
+        <v>248</v>
+      </c>
+      <c r="E26" s="45" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A27" s="43">
+        <v>23</v>
+      </c>
+      <c r="B27" s="44" t="s">
+        <v>199</v>
+      </c>
+      <c r="C27" s="44" t="s">
+        <v>203</v>
+      </c>
+      <c r="D27" s="42" t="s">
+        <v>250</v>
+      </c>
+      <c r="E27" s="42" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A28" s="46">
+        <v>24</v>
+      </c>
+      <c r="B28" s="47" t="s">
+        <v>199</v>
+      </c>
+      <c r="C28" s="47" t="s">
+        <v>203</v>
+      </c>
+      <c r="D28" s="45" t="s">
+        <v>252</v>
+      </c>
+      <c r="E28" s="45" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A29" s="43">
+        <v>25</v>
+      </c>
+      <c r="B29" s="44" t="s">
+        <v>199</v>
+      </c>
+      <c r="C29" s="44" t="s">
+        <v>203</v>
+      </c>
+      <c r="D29" s="42" t="s">
+        <v>254</v>
+      </c>
+      <c r="E29" s="42" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A30" s="46">
+        <v>26</v>
+      </c>
+      <c r="B30" s="47" t="s">
+        <v>199</v>
+      </c>
+      <c r="C30" s="47" t="s">
+        <v>200</v>
+      </c>
+      <c r="D30" s="45" t="s">
+        <v>256</v>
+      </c>
+      <c r="E30" s="45" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A31" s="43">
+        <v>27</v>
+      </c>
+      <c r="B31" s="44" t="s">
+        <v>199</v>
+      </c>
+      <c r="C31" s="44" t="s">
+        <v>215</v>
+      </c>
+      <c r="D31" s="42" t="s">
+        <v>258</v>
+      </c>
+      <c r="E31" s="42" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" s="46">
+        <v>28</v>
+      </c>
+      <c r="B32" s="47" t="s">
+        <v>214</v>
+      </c>
+      <c r="C32" s="47" t="s">
+        <v>200</v>
+      </c>
+      <c r="D32" s="45" t="s">
+        <v>260</v>
+      </c>
+      <c r="E32" s="45" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" s="43">
+        <v>29</v>
+      </c>
+      <c r="B33" s="44" t="s">
+        <v>199</v>
+      </c>
+      <c r="C33" s="44" t="s">
+        <v>200</v>
+      </c>
+      <c r="D33" s="42" t="s">
+        <v>262</v>
+      </c>
+      <c r="E33" s="42" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A34" s="46">
+        <v>30</v>
+      </c>
+      <c r="B34" s="47" t="s">
+        <v>199</v>
+      </c>
+      <c r="C34" s="47" t="s">
+        <v>203</v>
+      </c>
+      <c r="D34" s="45" t="s">
+        <v>264</v>
+      </c>
+      <c r="E34" s="45" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A35" s="43">
+        <v>31</v>
+      </c>
+      <c r="B35" s="44" t="s">
+        <v>199</v>
+      </c>
+      <c r="C35" s="44" t="s">
+        <v>203</v>
+      </c>
+      <c r="D35" s="42" t="s">
+        <v>266</v>
+      </c>
+      <c r="E35" s="42" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A36" s="46">
+        <v>32</v>
+      </c>
+      <c r="B36" s="47" t="s">
+        <v>199</v>
+      </c>
+      <c r="C36" s="47" t="s">
+        <v>203</v>
+      </c>
+      <c r="D36" s="45" t="s">
+        <v>268</v>
+      </c>
+      <c r="E36" s="45" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A37" s="43">
+        <v>33</v>
+      </c>
+      <c r="B37" s="44" t="s">
+        <v>199</v>
+      </c>
+      <c r="C37" s="44" t="s">
+        <v>203</v>
+      </c>
+      <c r="D37" s="42" t="s">
+        <v>270</v>
+      </c>
+      <c r="E37" s="42" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A38" s="46">
+        <v>34</v>
+      </c>
+      <c r="B38" s="47" t="s">
+        <v>199</v>
+      </c>
+      <c r="C38" s="47" t="s">
+        <v>200</v>
+      </c>
+      <c r="D38" s="45" t="s">
+        <v>272</v>
+      </c>
+      <c r="E38" s="45" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A39" s="43">
+        <v>35</v>
+      </c>
+      <c r="B39" s="44" t="s">
+        <v>199</v>
+      </c>
+      <c r="C39" s="44" t="s">
+        <v>203</v>
+      </c>
+      <c r="D39" s="42" t="s">
+        <v>274</v>
+      </c>
+      <c r="E39" s="42" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" s="53" t="s">
+        <v>276</v>
+      </c>
+      <c r="B41" s="54"/>
+      <c r="C41" s="54"/>
+      <c r="D41" s="54"/>
+      <c r="E41" s="54"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A41:E41"/>
+  </mergeCells>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECAE18B4-5A40-45A5-BDF9-F147409492E6}">
   <dimension ref="A1:C25"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.77734375" customWidth="1"/>
-    <col min="2" max="2" width="60.77734375" customWidth="1"/>
-    <col min="3" max="3" width="16.77734375" customWidth="1"/>
+    <col min="1" max="1" width="26.7109375" customWidth="1"/>
+    <col min="2" max="2" width="60.7109375" customWidth="1"/>
+    <col min="3" max="3" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="16" t="s">
+    <row r="1" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="65" t="s">
         <v>151</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-    </row>
-    <row r="2" spans="1:3" ht="7.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-    </row>
-    <row r="3" spans="1:3" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="8" t="s">
+      <c r="B1" s="65"/>
+      <c r="C1" s="65"/>
+    </row>
+    <row r="2" spans="1:3" ht="7.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+    </row>
+    <row r="3" spans="1:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="C3" s="8"/>
-    </row>
-    <row r="4" spans="1:3" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="11" t="s">
+      <c r="C3" s="3"/>
+    </row>
+    <row r="4" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="B4" s="54" t="s">
+      <c r="B4" s="67" t="s">
         <v>155</v>
       </c>
-      <c r="C4" s="53"/>
-    </row>
-    <row r="5" spans="1:3" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="14" t="s">
+      <c r="C4" s="68"/>
+    </row>
+    <row r="5" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="B5" s="55" t="s">
+      <c r="B5" s="69" t="s">
         <v>157</v>
       </c>
-      <c r="C5" s="12"/>
-    </row>
-    <row r="6" spans="1:3" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="11" t="s">
+      <c r="C5" s="60"/>
+    </row>
+    <row r="6" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="B6" s="54" t="s">
+      <c r="B6" s="67" t="s">
         <v>159</v>
       </c>
-      <c r="C6" s="12"/>
-    </row>
-    <row r="7" spans="1:3" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="14" t="s">
+      <c r="C6" s="60"/>
+    </row>
+    <row r="7" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="B7" s="55" t="s">
+      <c r="B7" s="69" t="s">
         <v>161</v>
       </c>
-      <c r="C7" s="12"/>
-    </row>
-    <row r="8" spans="1:3" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="11" t="s">
+      <c r="C7" s="60"/>
+    </row>
+    <row r="8" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="B8" s="54" t="s">
+      <c r="B8" s="67" t="s">
         <v>163</v>
       </c>
-      <c r="C8" s="12"/>
-    </row>
-    <row r="9" spans="1:3" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="14" t="s">
+      <c r="C8" s="60"/>
+    </row>
+    <row r="9" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
         <v>164</v>
       </c>
-      <c r="B9" s="55" t="s">
+      <c r="B9" s="69" t="s">
         <v>165</v>
       </c>
-      <c r="C9" s="12"/>
-    </row>
-    <row r="10" spans="1:3" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="11" t="s">
+      <c r="C9" s="60"/>
+    </row>
+    <row r="10" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="B10" s="54" t="s">
+      <c r="B10" s="67" t="s">
         <v>167</v>
       </c>
-      <c r="C10" s="12"/>
-    </row>
-    <row r="11" spans="1:3" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="14" t="s">
+      <c r="C10" s="60"/>
+    </row>
+    <row r="11" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="B11" s="55" t="s">
+      <c r="B11" s="69" t="s">
         <v>169</v>
       </c>
-      <c r="C11" s="12"/>
-    </row>
-    <row r="12" spans="1:3" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="11" t="s">
+      <c r="C11" s="60"/>
+    </row>
+    <row r="12" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="B12" s="54" t="s">
+      <c r="B12" s="67" t="s">
         <v>171</v>
       </c>
-      <c r="C12" s="12"/>
-    </row>
-    <row r="13" spans="1:3" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="14" t="s">
+      <c r="C12" s="60"/>
+    </row>
+    <row r="13" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
         <v>172</v>
       </c>
-      <c r="B13" s="55" t="s">
+      <c r="B13" s="69" t="s">
         <v>173</v>
       </c>
-      <c r="C13" s="12"/>
-    </row>
-    <row r="16" spans="1:3" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="7" t="s">
+      <c r="C13" s="60"/>
+    </row>
+    <row r="16" spans="1:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="61" t="s">
         <v>174</v>
       </c>
-      <c r="B16" s="7"/>
-      <c r="C16" s="7"/>
-    </row>
-    <row r="17" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="8" t="s">
+      <c r="B16" s="61"/>
+      <c r="C16" s="61"/>
+    </row>
+    <row r="17" spans="1:3" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="62" t="s">
         <v>25</v>
       </c>
-      <c r="C17" s="9"/>
-    </row>
-    <row r="18" spans="1:3" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="11" t="s">
+      <c r="C17" s="63"/>
+    </row>
+    <row r="18" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="B18" s="54" t="s">
+      <c r="B18" s="67" t="s">
         <v>177</v>
       </c>
-      <c r="C18" s="12"/>
-    </row>
-    <row r="19" spans="1:3" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="14" t="s">
+      <c r="C18" s="60"/>
+    </row>
+    <row r="19" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="B19" s="55" t="s">
+      <c r="B19" s="69" t="s">
         <v>179</v>
       </c>
-      <c r="C19" s="12"/>
-    </row>
-    <row r="20" spans="1:3" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="11" t="s">
+      <c r="C19" s="60"/>
+    </row>
+    <row r="20" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="B20" s="54" t="s">
+      <c r="B20" s="67" t="s">
         <v>181</v>
       </c>
-      <c r="C20" s="12"/>
-    </row>
-    <row r="21" spans="1:3" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="14" t="s">
+      <c r="C20" s="60"/>
+    </row>
+    <row r="21" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="6" t="s">
         <v>182</v>
       </c>
-      <c r="B21" s="55" t="s">
+      <c r="B21" s="69" t="s">
         <v>183</v>
       </c>
-      <c r="C21" s="12"/>
-    </row>
-    <row r="22" spans="1:3" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="11" t="s">
+      <c r="C21" s="60"/>
+    </row>
+    <row r="22" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
         <v>184</v>
       </c>
-      <c r="B22" s="54" t="s">
+      <c r="B22" s="67" t="s">
         <v>185</v>
       </c>
-      <c r="C22" s="12"/>
-    </row>
-    <row r="23" spans="1:3" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="14" t="s">
+      <c r="C22" s="60"/>
+    </row>
+    <row r="23" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="B23" s="55" t="s">
+      <c r="B23" s="69" t="s">
         <v>187</v>
       </c>
-      <c r="C23" s="12"/>
-    </row>
-    <row r="24" spans="1:3" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="11" t="s">
+      <c r="C23" s="60"/>
+    </row>
+    <row r="24" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="B24" s="54" t="s">
+      <c r="B24" s="67" t="s">
         <v>189</v>
       </c>
-      <c r="C24" s="12"/>
-    </row>
-    <row r="25" spans="1:3" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="14" t="s">
+      <c r="C24" s="60"/>
+    </row>
+    <row r="25" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="6" t="s">
         <v>190</v>
       </c>
-      <c r="B25" s="55" t="s">
+      <c r="B25" s="69" t="s">
         <v>191</v>
       </c>
-      <c r="C25" s="12"/>
+      <c r="C25" s="60"/>
     </row>
   </sheetData>
   <mergeCells count="21">
@@ -2374,11 +3394,6 @@
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B13:C13"/>
     <mergeCell ref="A16:C16"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="B4:C4"/>
@@ -2386,6 +3401,11 @@
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B13:C13"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: atualizar documentos de backup para v4.2 (auditoria)
Sincroniza os artefatos de integridade do projeto com o estado real após a
auditoria de 9 lotes:

- CONTEXTO_CLAUDE.md (handoff): versão v4.2, ~5310 linhas, sw.js network-first;
  nova seção 17 registrando os 9 lotes da auditoria e as decisões em aberto;
  correções factuais (R07 "próximo a", R25 "Máquinas e Equipamentos", equipe 45,
  helpers esc()/fetchComTimeout); nota sobre mudanças no autoSyncComPDF.
- APR_REMO_Documentacao.html: versão 4.2, contagens e datas atualizadas,
  linha de changelog da auditoria + entrada de mapa/logo.
- APR_REMO_Historico_Projeto.xlsx: Visão Geral (v4.2, 03/07/2026), 11 linhas
  no Histórico de Commits (9 lotes + mapa/logo), Banco de Riscos R07/R25.
  Backup espelhado em Documentos/Claude/APR_REMO.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/APR_REMO_Historico_Projeto.xlsx
+++ b/APR_REMO_Historico_Projeto.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Remo Engenharia\Desktop\apr\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C376562-E6C1-4CF9-87BA-905C9768F8CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAF8CC94-C36D-49FA-A3BC-F523FEA7F831}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="4" xr2:uid="{E8D2854C-CAA7-4AC3-9D15-57F2C505D09B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="302">
   <si>
     <t>SISTEMA APR DIGITAL — REMO ENGENHARIA</t>
   </si>
@@ -68,9 +68,6 @@
     <t>Arquivo</t>
   </si>
   <si>
-    <t>index.html  (single-file PWA, 4421 linhas)</t>
-  </si>
-  <si>
     <t>URL pública</t>
   </si>
   <si>
@@ -689,9 +686,6 @@
     <t>Crítica</t>
   </si>
   <si>
-    <t>Trabalho próx. a Circuitos Energizados</t>
-  </si>
-  <si>
     <t>Manter distâncias de segurança dos pontos energizados. 345 kV Distância mínima de aproximação: 3,5 metros - 138 kV Distância mínima de aproximação: 1,5 metros.</t>
   </si>
   <si>
@@ -803,9 +797,6 @@
     <t>Atentar ao trajeto perante veículos e máquinas. Contato visual com motorista e sinaleiro.</t>
   </si>
   <si>
-    <t>Máquinas sem Proteção</t>
-  </si>
-  <si>
     <t>Verificar proteções de máquinas conforme NR-12 antes de operar. Nunca remover proteções.</t>
   </si>
   <si>
@@ -872,13 +863,97 @@
     <t>* Riscos 07, 09 e 13 atualizados em 18/06/2026 — Observações padrão incluídas / Máscara UV removida do R13.</t>
   </si>
   <si>
-    <t>18/06/2026</t>
+    <t>index.html  (single-file PWA, 5310 linhas) + sw.js</t>
+  </si>
+  <si>
+    <t>v4.2 Lote 9</t>
+  </si>
+  <si>
+    <t>Dados: grafia Caminhao Munck, checklist Motoserra sem 'Trado de perfuracao', perigo 'Queda de objetos' remapeado ao risco 33. Versao do app v4.2.</t>
+  </si>
+  <si>
+    <t>v4.2 Lote 8</t>
+  </si>
+  <si>
+    <t>Acessibilidade: zoom liberado (WCAG 1.4.4), alvo de toque 44px nos cards .ac, dark mode corrigido (dot ativo, titulos do Resumo), placeholders 4.5:1, prefers-reduced-motion.</t>
+  </si>
+  <si>
+    <t>v4.2 Lote 7</t>
+  </si>
+  <si>
+    <t>PWA: service worker network-first (equipe sempre na versao mais recente online), cache versionado apr-remo-v2, manifesto unico (removido estatico corrompido).</t>
+  </si>
+  <si>
+    <t>v4.2 Lote 6</t>
+  </si>
+  <si>
+    <t>Impressao: page-break-inside:avoid em linhas de tabela/assinaturas, modo escuro nao vaza mais para documento/PDF, QR do cabecalho com crossorigin.</t>
+  </si>
+  <si>
+    <t>v4.2 Lote 5</t>
+  </si>
+  <si>
+    <t>Sync: badge honesto 'Enviado ao Drive' (no-cors nao confirma gravacao), timeout 30s, guarda 20MB no PDF, try/catch no localStorage (apr_favs nao derruba mais o app).</t>
+  </si>
+  <si>
+    <t>v4.2 Lote 4</t>
+  </si>
+  <si>
+    <t>Seguranca: funcao esc() em ~20 pontos de interpolacao (XSS e '&lt;' em observacoes nao quebram o documento), URL do Drive exige /macros/.</t>
+  </si>
+  <si>
+    <t>v4.2 Lote 3</t>
+  </si>
+  <si>
+    <t>Fluxo: validar() cobre Etapas 3/4 (APR nao sai sem risco avaliado nem sem equipe), dots corretos na tela final, logout com reset completo do rascunho.</t>
+  </si>
+  <si>
+    <t>v4.2 Lote 2</t>
+  </si>
+  <si>
+    <t>Catalogo: risco 7 'Trabalho proximo a Circuitos Energizados' selecionavel nas ~34 fases (antes 'prox.' impedia o match), risco 25 renomeado, matcher normalizado, nivel da fase = pior risco (nao media).</t>
+  </si>
+  <si>
+    <t>v4.2 Lote 1</t>
+  </si>
+  <si>
+    <t>Estado da Etapa 3: 8 bugs SEL_RISCOS corrigidos (vazamento de riscos entre atividades, corrupcao de templates persistidos, complementos perdidos, chaves orfas).</t>
+  </si>
+  <si>
+    <t>20/06/2026</t>
+  </si>
+  <si>
+    <t>v4.1 Logo</t>
+  </si>
+  <si>
+    <t>Efeito degrade azul-verde no logo REMO ao avancar etapas; logo ampliado para 48px.</t>
+  </si>
+  <si>
+    <t>19/06/2026</t>
+  </si>
+  <si>
+    <t>v4.1 Mapa</t>
+  </si>
+  <si>
+    <t>Mapa SVG estatico de rota de emergencia (obra ate hospital de Rifaina) + QR code base64 na ultima folha impressa. Substitui Leaflet interativo (inadequado para impressao).</t>
+  </si>
+  <si>
+    <t>Trabalho próximo a Circuitos Energizados</t>
+  </si>
+  <si>
+    <t>Máquinas e Equipamentos sem Proteção</t>
+  </si>
+  <si>
+    <t>03/07/2026</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd/mm/\y\y\y\y"/>
+  </numFmts>
   <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1146,7 +1221,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1215,9 +1290,6 @@
     <xf numFmtId="0" fontId="10" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="7" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1294,6 +1366,9 @@
     <xf numFmtId="0" fontId="17" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1303,34 +1378,37 @@
     <xf numFmtId="0" fontId="18" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="4" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1338,14 +1416,17 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1670,18 +1751,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="63" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="57"/>
-      <c r="C1" s="57"/>
+      <c r="B1" s="63"/>
+      <c r="C1" s="63"/>
     </row>
     <row r="2" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="64" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="58"/>
-      <c r="C2" s="58"/>
+      <c r="B2" s="64"/>
+      <c r="C2" s="64"/>
     </row>
     <row r="3" spans="1:3" ht="7.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -1692,200 +1773,212 @@
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="55" t="s">
+      <c r="B4" s="57" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="56"/>
+      <c r="C4" s="58"/>
     </row>
     <row r="5" spans="1:3" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="55" t="s">
+      <c r="B5" s="57" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="56"/>
+      <c r="C5" s="58"/>
     </row>
     <row r="6" spans="1:3" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="55" t="s">
+      <c r="B6" s="57" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="56"/>
+      <c r="C6" s="58"/>
     </row>
     <row r="7" spans="1:3" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="55" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7" s="56"/>
+      <c r="B7" s="57" t="s">
+        <v>274</v>
+      </c>
+      <c r="C7" s="58"/>
     </row>
     <row r="8" spans="1:3" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="57" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="55" t="s">
-        <v>11</v>
-      </c>
-      <c r="C8" s="56"/>
+      <c r="C8" s="58"/>
     </row>
     <row r="9" spans="1:3" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="57" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="55" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" s="56"/>
+      <c r="C9" s="58"/>
     </row>
     <row r="10" spans="1:3" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" s="55">
-        <v>4.0999999999999996</v>
-      </c>
-      <c r="C10" s="56"/>
+        <v>13</v>
+      </c>
+      <c r="B10" s="57">
+        <v>4.2</v>
+      </c>
+      <c r="C10" s="58"/>
     </row>
     <row r="11" spans="1:3" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="57" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="55" t="s">
-        <v>16</v>
-      </c>
-      <c r="C11" s="56"/>
+      <c r="C11" s="58"/>
     </row>
     <row r="12" spans="1:3" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B12" s="55" t="s">
-        <v>277</v>
-      </c>
-      <c r="C12" s="56"/>
+        <v>16</v>
+      </c>
+      <c r="B12" s="65">
+        <v>46088</v>
+      </c>
+      <c r="C12" s="58"/>
     </row>
     <row r="13" spans="1:3" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13" s="57" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="55" t="s">
-        <v>20</v>
-      </c>
-      <c r="C13" s="56"/>
+      <c r="C13" s="58"/>
     </row>
     <row r="14" spans="1:3" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="57" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="55" t="s">
+      <c r="C14" s="58"/>
+    </row>
+    <row r="16" spans="1:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="59" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="56"/>
-    </row>
-    <row r="16" spans="1:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="61" t="s">
-        <v>23</v>
-      </c>
-      <c r="B16" s="61"/>
-      <c r="C16" s="61"/>
+      <c r="B16" s="59"/>
+      <c r="C16" s="59"/>
     </row>
     <row r="17" spans="1:3" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17" s="60" t="s">
         <v>24</v>
       </c>
-      <c r="B17" s="62" t="s">
-        <v>25</v>
-      </c>
-      <c r="C17" s="63"/>
+      <c r="C17" s="61"/>
     </row>
     <row r="18" spans="1:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B18" s="55" t="s">
         <v>26</v>
       </c>
-      <c r="B18" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="C18" s="60"/>
+      <c r="C18" s="56"/>
     </row>
     <row r="19" spans="1:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19" s="62" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="64" t="s">
-        <v>29</v>
-      </c>
-      <c r="C19" s="60"/>
+      <c r="C19" s="56"/>
     </row>
     <row r="20" spans="1:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B20" s="55" t="s">
         <v>30</v>
       </c>
-      <c r="B20" s="59" t="s">
-        <v>31</v>
-      </c>
-      <c r="C20" s="60"/>
+      <c r="C20" s="56"/>
     </row>
     <row r="21" spans="1:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B21" s="62" t="s">
         <v>32</v>
       </c>
-      <c r="B21" s="64" t="s">
-        <v>33</v>
-      </c>
-      <c r="C21" s="60"/>
+      <c r="C21" s="56"/>
     </row>
     <row r="22" spans="1:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B22" s="55" t="s">
         <v>34</v>
       </c>
-      <c r="B22" s="59" t="s">
-        <v>35</v>
-      </c>
-      <c r="C22" s="60"/>
+      <c r="C22" s="56"/>
     </row>
     <row r="23" spans="1:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B23" s="62" t="s">
         <v>36</v>
       </c>
-      <c r="B23" s="64" t="s">
-        <v>37</v>
-      </c>
-      <c r="C23" s="60"/>
+      <c r="C23" s="56"/>
     </row>
     <row r="24" spans="1:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B24" s="55" t="s">
         <v>38</v>
       </c>
-      <c r="B24" s="59" t="s">
-        <v>39</v>
-      </c>
-      <c r="C24" s="60"/>
+      <c r="C24" s="56"/>
     </row>
     <row r="25" spans="1:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B25" s="62" t="s">
         <v>40</v>
       </c>
-      <c r="B25" s="64" t="s">
-        <v>41</v>
-      </c>
-      <c r="C25" s="60"/>
+      <c r="C25" s="56"/>
     </row>
     <row r="26" spans="1:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B26" s="55" t="s">
         <v>42</v>
       </c>
-      <c r="B26" s="59" t="s">
-        <v>43</v>
-      </c>
-      <c r="C26" s="60"/>
+      <c r="C26" s="56"/>
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
     <mergeCell ref="B26:C26"/>
     <mergeCell ref="B14:C14"/>
     <mergeCell ref="A16:C16"/>
@@ -1898,18 +1991,6 @@
     <mergeCell ref="B23:C23"/>
     <mergeCell ref="B24:C24"/>
     <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
@@ -1917,7 +1998,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8EE7C958-1583-4AC7-AE30-B3B76C482C0D}">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.7109375" customWidth="1"/>
@@ -1927,12 +2008,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="65" t="s">
-        <v>44</v>
-      </c>
-      <c r="B1" s="65"/>
-      <c r="C1" s="65"/>
-      <c r="D1" s="65"/>
+      <c r="A1" s="66" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
     </row>
     <row r="2" spans="1:4" ht="7.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
@@ -1942,156 +2023,310 @@
     </row>
     <row r="3" spans="1:4" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D3" s="3" t="s">
+    </row>
+    <row r="4" spans="1:4" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="71" t="s">
+        <v>301</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="71" t="s">
+        <v>301</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="71" t="s">
+        <v>301</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="71" t="s">
+        <v>301</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="71" t="s">
+        <v>301</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="71" t="s">
+        <v>301</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="71" t="s">
+        <v>301</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="71" t="s">
+        <v>301</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>290</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="71" t="s">
+        <v>301</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="71" t="s">
+        <v>293</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="71" t="s">
+        <v>296</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" s="9" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" s="9" t="s">
+      <c r="C15" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="D15" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="D4" s="11" t="s">
+    </row>
+    <row r="16" spans="1:4" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="8" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
+      <c r="B16" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="C16" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="D16" s="11" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="D5" s="11" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="12" t="s">
+      <c r="B17" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="C17" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="D17" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="D6" s="15" t="s">
+    </row>
+    <row r="18" spans="1:4" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B18" s="13" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="B7" s="13" t="s">
+      <c r="C18" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="D18" s="15" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="B19" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="D7" s="15" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="B8" s="17" t="s">
+      <c r="C19" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="D19" s="19" t="s">
         <v>62</v>
       </c>
-      <c r="D8" s="19" t="s">
+    </row>
+    <row r="20" spans="1:4" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="B20" s="17" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="B9" s="17" t="s">
+      <c r="C20" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="D20" s="19" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="D9" s="19" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="20" t="s">
+      <c r="B21" s="21" t="s">
         <v>66</v>
       </c>
-      <c r="B10" s="21" t="s">
+      <c r="C21" s="22" t="s">
         <v>67</v>
       </c>
-      <c r="C10" s="22" t="s">
+      <c r="D21" s="23" t="s">
         <v>68</v>
       </c>
-      <c r="D10" s="23" t="s">
+    </row>
+    <row r="22" spans="1:4" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="50">
+        <v>46178</v>
+      </c>
+      <c r="B22" s="24" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="24">
-        <v>46178</v>
-      </c>
-      <c r="B11" s="25" t="s">
+      <c r="C22" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="C11" s="26" t="s">
+      <c r="D22" s="26" t="s">
         <v>71</v>
       </c>
-      <c r="D11" s="27" t="s">
+    </row>
+    <row r="23" spans="1:4" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="27" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="28" t="s">
+      <c r="B23" s="28" t="s">
         <v>73</v>
       </c>
-      <c r="B12" s="29" t="s">
+      <c r="C23" s="29" t="s">
         <v>74</v>
       </c>
-      <c r="C12" s="30" t="s">
+      <c r="D23" s="30" t="s">
         <v>75</v>
       </c>
-      <c r="D12" s="31" t="s">
+    </row>
+    <row r="24" spans="1:4" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="31" t="s">
+        <v>15</v>
+      </c>
+      <c r="B24" s="32" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="32" t="s">
-        <v>16</v>
-      </c>
-      <c r="B13" s="33" t="s">
+      <c r="C24" s="33" t="s">
         <v>77</v>
       </c>
-      <c r="C13" s="34" t="s">
+      <c r="D24" s="34" t="s">
         <v>78</v>
-      </c>
-      <c r="D13" s="35" t="s">
-        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -2113,11 +2348,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="65" t="s">
-        <v>80</v>
-      </c>
-      <c r="B1" s="65"/>
-      <c r="C1" s="65"/>
+      <c r="A1" s="66" t="s">
+        <v>79</v>
+      </c>
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
     </row>
     <row r="2" spans="1:3" ht="7.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
@@ -2126,200 +2361,200 @@
     </row>
     <row r="3" spans="1:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>82</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="C4" s="35" t="s">
         <v>85</v>
-      </c>
-      <c r="C4" s="36" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B5" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="B5" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="C5" s="37" t="s">
-        <v>86</v>
+      <c r="C5" s="36" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="B6" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="C6" s="36" t="s">
-        <v>86</v>
+      <c r="C6" s="35" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="B7" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="B7" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="C7" s="37" t="s">
-        <v>86</v>
+      <c r="C7" s="36" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="B8" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="C8" s="36" t="s">
-        <v>86</v>
+      <c r="C8" s="35" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="B9" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="B9" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="C9" s="37" t="s">
-        <v>86</v>
+      <c r="C9" s="36" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B10" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="B10" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="C10" s="36" t="s">
-        <v>86</v>
+      <c r="C10" s="35" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="B11" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="B11" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="C11" s="37" t="s">
-        <v>86</v>
+      <c r="C11" s="36" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="B12" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="B12" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="C12" s="36" t="s">
-        <v>86</v>
+      <c r="C12" s="35" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="B13" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="B13" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="C13" s="37" t="s">
-        <v>86</v>
+      <c r="C13" s="36" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B14" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="B14" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="C14" s="36" t="s">
-        <v>86</v>
+      <c r="C14" s="35" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B15" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="B15" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="C15" s="37" t="s">
-        <v>86</v>
+      <c r="C15" s="36" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="B16" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="B16" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="C16" s="36" t="s">
-        <v>86</v>
+      <c r="C16" s="35" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B17" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="B17" s="7" t="s">
-        <v>112</v>
-      </c>
-      <c r="C17" s="37" t="s">
-        <v>86</v>
+      <c r="C17" s="36" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B18" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="B18" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="C18" s="36" t="s">
-        <v>86</v>
+      <c r="C18" s="35" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="B19" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="B19" s="7" t="s">
-        <v>116</v>
-      </c>
-      <c r="C19" s="37" t="s">
-        <v>86</v>
+      <c r="C19" s="36" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="B20" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="B20" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="C20" s="36" t="s">
-        <v>86</v>
+      <c r="C20" s="35" t="s">
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -2342,12 +2577,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="65" t="s">
-        <v>119</v>
-      </c>
-      <c r="B1" s="65"/>
-      <c r="C1" s="65"/>
-      <c r="D1" s="65"/>
+      <c r="A1" s="66" t="s">
+        <v>118</v>
+      </c>
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
     </row>
     <row r="2" spans="1:4" ht="7.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
@@ -2357,151 +2592,151 @@
     </row>
     <row r="3" spans="1:4" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>121</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="B4" s="37">
+        <v>32</v>
+      </c>
+      <c r="C4" s="38" t="s">
         <v>123</v>
       </c>
-      <c r="B4" s="38">
-        <v>32</v>
-      </c>
-      <c r="C4" s="39" t="s">
+      <c r="D4" s="38" t="s">
         <v>124</v>
-      </c>
-      <c r="D4" s="39" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="B5" s="39">
+        <v>35</v>
+      </c>
+      <c r="C5" s="25" t="s">
         <v>126</v>
       </c>
-      <c r="B5" s="40">
-        <v>35</v>
-      </c>
-      <c r="C5" s="26" t="s">
+      <c r="D5" s="25" t="s">
         <v>127</v>
-      </c>
-      <c r="D5" s="26" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="B6" s="37">
+        <v>46</v>
+      </c>
+      <c r="C6" s="38" t="s">
         <v>129</v>
       </c>
-      <c r="B6" s="38">
-        <v>46</v>
-      </c>
-      <c r="C6" s="39" t="s">
+      <c r="D6" s="38" t="s">
         <v>130</v>
-      </c>
-      <c r="D6" s="39" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="B7" s="39">
+        <v>7</v>
+      </c>
+      <c r="C7" s="25" t="s">
         <v>132</v>
       </c>
-      <c r="B7" s="40">
-        <v>7</v>
-      </c>
-      <c r="C7" s="26" t="s">
+      <c r="D7" s="25" t="s">
         <v>133</v>
-      </c>
-      <c r="D7" s="26" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="B8" s="37" t="s">
         <v>135</v>
       </c>
-      <c r="B8" s="38" t="s">
+      <c r="C8" s="38" t="s">
         <v>136</v>
       </c>
-      <c r="C8" s="39" t="s">
+      <c r="D8" s="38" t="s">
         <v>137</v>
-      </c>
-      <c r="D8" s="39" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="B9" s="39">
+        <v>33</v>
+      </c>
+      <c r="C9" s="25" t="s">
         <v>139</v>
       </c>
-      <c r="B9" s="40">
-        <v>33</v>
-      </c>
-      <c r="C9" s="26" t="s">
+      <c r="D9" s="25" t="s">
         <v>140</v>
-      </c>
-      <c r="D9" s="26" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="B10" s="37">
+        <v>14</v>
+      </c>
+      <c r="C10" s="38" t="s">
         <v>142</v>
       </c>
-      <c r="B10" s="38">
-        <v>14</v>
-      </c>
-      <c r="C10" s="39" t="s">
+      <c r="D10" s="38" t="s">
         <v>143</v>
-      </c>
-      <c r="D10" s="39" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="B11" s="39">
+        <v>28</v>
+      </c>
+      <c r="C11" s="25" t="s">
         <v>145</v>
       </c>
-      <c r="B11" s="40">
-        <v>28</v>
-      </c>
-      <c r="C11" s="26" t="s">
-        <v>146</v>
-      </c>
-      <c r="D11" s="26" t="s">
-        <v>144</v>
+      <c r="D11" s="25" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="B12" s="37">
+        <v>2</v>
+      </c>
+      <c r="C12" s="38" t="s">
         <v>147</v>
       </c>
-      <c r="B12" s="38">
-        <v>2</v>
-      </c>
-      <c r="C12" s="39" t="s">
+      <c r="D12" s="38" t="s">
         <v>148</v>
       </c>
-      <c r="D12" s="39" t="s">
+    </row>
+    <row r="14" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="67" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="66" t="s">
-        <v>150</v>
-      </c>
-      <c r="B14" s="66"/>
-      <c r="C14" s="66"/>
-      <c r="D14" s="66"/>
+      <c r="B14" s="67"/>
+      <c r="C14" s="67"/>
+      <c r="D14" s="67"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2526,7 +2761,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="51" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B1" s="51"/>
       <c r="C1" s="51"/>
@@ -2535,7 +2770,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="52" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B2" s="52"/>
       <c r="C2" s="52"/>
@@ -2544,620 +2779,620 @@
     </row>
     <row r="3" spans="1:5" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="41" t="s">
+      <c r="A4" s="40" t="s">
+        <v>193</v>
+      </c>
+      <c r="B4" s="40" t="s">
         <v>194</v>
       </c>
-      <c r="B4" s="41" t="s">
+      <c r="C4" s="40" t="s">
         <v>195</v>
       </c>
-      <c r="C4" s="41" t="s">
+      <c r="D4" s="40" t="s">
         <v>196</v>
       </c>
-      <c r="D4" s="41" t="s">
+      <c r="E4" s="40" t="s">
         <v>197</v>
       </c>
-      <c r="E4" s="41" t="s">
+    </row>
+    <row r="5" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="42">
+        <v>1</v>
+      </c>
+      <c r="B5" s="43" t="s">
         <v>198</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="43">
-        <v>1</v>
-      </c>
-      <c r="B5" s="44" t="s">
+      <c r="C5" s="43" t="s">
         <v>199</v>
       </c>
-      <c r="C5" s="44" t="s">
+      <c r="D5" s="41" t="s">
         <v>200</v>
       </c>
-      <c r="D5" s="42" t="s">
+      <c r="E5" s="41" t="s">
         <v>201</v>
       </c>
-      <c r="E5" s="42" t="s">
+    </row>
+    <row r="6" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="45">
+        <v>2</v>
+      </c>
+      <c r="B6" s="46" t="s">
+        <v>198</v>
+      </c>
+      <c r="C6" s="46" t="s">
         <v>202</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="46">
-        <v>2</v>
-      </c>
-      <c r="B6" s="47" t="s">
+      <c r="D6" s="44" t="s">
+        <v>203</v>
+      </c>
+      <c r="E6" s="44" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="42">
+        <v>3</v>
+      </c>
+      <c r="B7" s="43" t="s">
+        <v>198</v>
+      </c>
+      <c r="C7" s="43" t="s">
         <v>199</v>
       </c>
-      <c r="C6" s="47" t="s">
-        <v>203</v>
-      </c>
-      <c r="D6" s="45" t="s">
-        <v>204</v>
-      </c>
-      <c r="E6" s="45" t="s">
+      <c r="D7" s="41" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="43">
-        <v>3</v>
-      </c>
-      <c r="B7" s="44" t="s">
+      <c r="E7" s="41" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="45">
+        <v>4</v>
+      </c>
+      <c r="B8" s="46" t="s">
+        <v>198</v>
+      </c>
+      <c r="C8" s="46" t="s">
         <v>199</v>
       </c>
-      <c r="C7" s="44" t="s">
-        <v>200</v>
-      </c>
-      <c r="D7" s="42" t="s">
-        <v>206</v>
-      </c>
-      <c r="E7" s="42" t="s">
+      <c r="D8" s="44" t="s">
         <v>207</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="46">
-        <v>4</v>
-      </c>
-      <c r="B8" s="47" t="s">
+      <c r="E8" s="44" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="42">
+        <v>5</v>
+      </c>
+      <c r="B9" s="43" t="s">
+        <v>198</v>
+      </c>
+      <c r="C9" s="43" t="s">
+        <v>202</v>
+      </c>
+      <c r="D9" s="41" t="s">
+        <v>209</v>
+      </c>
+      <c r="E9" s="41" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="45">
+        <v>6</v>
+      </c>
+      <c r="B10" s="46" t="s">
+        <v>198</v>
+      </c>
+      <c r="C10" s="46" t="s">
         <v>199</v>
       </c>
-      <c r="C8" s="47" t="s">
-        <v>200</v>
-      </c>
-      <c r="D8" s="45" t="s">
-        <v>208</v>
-      </c>
-      <c r="E8" s="45" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A9" s="43">
-        <v>5</v>
-      </c>
-      <c r="B9" s="44" t="s">
+      <c r="D10" s="44" t="s">
+        <v>211</v>
+      </c>
+      <c r="E10" s="44" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="49">
+        <v>7</v>
+      </c>
+      <c r="B11" s="48" t="s">
+        <v>213</v>
+      </c>
+      <c r="C11" s="48" t="s">
+        <v>214</v>
+      </c>
+      <c r="D11" s="47" t="s">
+        <v>299</v>
+      </c>
+      <c r="E11" s="47" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="45">
+        <v>8</v>
+      </c>
+      <c r="B12" s="46" t="s">
+        <v>198</v>
+      </c>
+      <c r="C12" s="46" t="s">
+        <v>214</v>
+      </c>
+      <c r="D12" s="44" t="s">
+        <v>216</v>
+      </c>
+      <c r="E12" s="44" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A13" s="49">
+        <v>9</v>
+      </c>
+      <c r="B13" s="48" t="s">
+        <v>213</v>
+      </c>
+      <c r="C13" s="48" t="s">
+        <v>202</v>
+      </c>
+      <c r="D13" s="47" t="s">
+        <v>218</v>
+      </c>
+      <c r="E13" s="47" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="45">
+        <v>10</v>
+      </c>
+      <c r="B14" s="46" t="s">
+        <v>198</v>
+      </c>
+      <c r="C14" s="46" t="s">
+        <v>202</v>
+      </c>
+      <c r="D14" s="44" t="s">
+        <v>220</v>
+      </c>
+      <c r="E14" s="44" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A15" s="42">
+        <v>11</v>
+      </c>
+      <c r="B15" s="43" t="s">
+        <v>198</v>
+      </c>
+      <c r="C15" s="43" t="s">
+        <v>214</v>
+      </c>
+      <c r="D15" s="41" t="s">
+        <v>222</v>
+      </c>
+      <c r="E15" s="41" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="45">
+        <v>12</v>
+      </c>
+      <c r="B16" s="46" t="s">
+        <v>213</v>
+      </c>
+      <c r="C16" s="46" t="s">
         <v>199</v>
       </c>
-      <c r="C9" s="44" t="s">
-        <v>203</v>
-      </c>
-      <c r="D9" s="42" t="s">
-        <v>210</v>
-      </c>
-      <c r="E9" s="42" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="46">
-        <v>6</v>
-      </c>
-      <c r="B10" s="47" t="s">
+      <c r="D16" s="44" t="s">
+        <v>224</v>
+      </c>
+      <c r="E16" s="44" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="49">
+        <v>13</v>
+      </c>
+      <c r="B17" s="48" t="s">
+        <v>213</v>
+      </c>
+      <c r="C17" s="48" t="s">
+        <v>226</v>
+      </c>
+      <c r="D17" s="47" t="s">
+        <v>227</v>
+      </c>
+      <c r="E17" s="47" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="45">
+        <v>14</v>
+      </c>
+      <c r="B18" s="46" t="s">
+        <v>198</v>
+      </c>
+      <c r="C18" s="46" t="s">
+        <v>214</v>
+      </c>
+      <c r="D18" s="44" t="s">
+        <v>229</v>
+      </c>
+      <c r="E18" s="44" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A19" s="42">
+        <v>15</v>
+      </c>
+      <c r="B19" s="43" t="s">
+        <v>198</v>
+      </c>
+      <c r="C19" s="43" t="s">
         <v>199</v>
       </c>
-      <c r="C10" s="47" t="s">
-        <v>200</v>
-      </c>
-      <c r="D10" s="45" t="s">
-        <v>212</v>
-      </c>
-      <c r="E10" s="45" t="s">
+      <c r="D19" s="41" t="s">
+        <v>231</v>
+      </c>
+      <c r="E19" s="41" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="45">
+        <v>16</v>
+      </c>
+      <c r="B20" s="46" t="s">
+        <v>198</v>
+      </c>
+      <c r="C20" s="46" t="s">
+        <v>199</v>
+      </c>
+      <c r="D20" s="44" t="s">
+        <v>233</v>
+      </c>
+      <c r="E20" s="44" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="42">
+        <v>17</v>
+      </c>
+      <c r="B21" s="43" t="s">
+        <v>198</v>
+      </c>
+      <c r="C21" s="43" t="s">
+        <v>214</v>
+      </c>
+      <c r="D21" s="41" t="s">
+        <v>235</v>
+      </c>
+      <c r="E21" s="41" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="45">
+        <v>18</v>
+      </c>
+      <c r="B22" s="46" t="s">
         <v>213</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="50">
-        <v>7</v>
-      </c>
-      <c r="B11" s="49" t="s">
+      <c r="C22" s="46" t="s">
+        <v>226</v>
+      </c>
+      <c r="D22" s="44" t="s">
+        <v>237</v>
+      </c>
+      <c r="E22" s="44" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="42">
+        <v>19</v>
+      </c>
+      <c r="B23" s="43" t="s">
+        <v>213</v>
+      </c>
+      <c r="C23" s="43" t="s">
+        <v>199</v>
+      </c>
+      <c r="D23" s="41" t="s">
+        <v>239</v>
+      </c>
+      <c r="E23" s="41" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="45">
+        <v>20</v>
+      </c>
+      <c r="B24" s="46" t="s">
+        <v>198</v>
+      </c>
+      <c r="C24" s="46" t="s">
+        <v>202</v>
+      </c>
+      <c r="D24" s="44" t="s">
+        <v>241</v>
+      </c>
+      <c r="E24" s="44" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A25" s="42">
+        <v>21</v>
+      </c>
+      <c r="B25" s="43" t="s">
+        <v>198</v>
+      </c>
+      <c r="C25" s="43" t="s">
+        <v>202</v>
+      </c>
+      <c r="D25" s="41" t="s">
+        <v>243</v>
+      </c>
+      <c r="E25" s="41" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A26" s="45">
+        <v>22</v>
+      </c>
+      <c r="B26" s="46" t="s">
+        <v>245</v>
+      </c>
+      <c r="C26" s="46" t="s">
+        <v>199</v>
+      </c>
+      <c r="D26" s="44" t="s">
+        <v>246</v>
+      </c>
+      <c r="E26" s="44" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A27" s="42">
+        <v>23</v>
+      </c>
+      <c r="B27" s="43" t="s">
+        <v>198</v>
+      </c>
+      <c r="C27" s="43" t="s">
+        <v>202</v>
+      </c>
+      <c r="D27" s="41" t="s">
+        <v>248</v>
+      </c>
+      <c r="E27" s="41" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A28" s="45">
+        <v>24</v>
+      </c>
+      <c r="B28" s="46" t="s">
+        <v>198</v>
+      </c>
+      <c r="C28" s="46" t="s">
+        <v>202</v>
+      </c>
+      <c r="D28" s="44" t="s">
+        <v>250</v>
+      </c>
+      <c r="E28" s="44" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A29" s="42">
+        <v>25</v>
+      </c>
+      <c r="B29" s="43" t="s">
+        <v>198</v>
+      </c>
+      <c r="C29" s="43" t="s">
+        <v>202</v>
+      </c>
+      <c r="D29" s="41" t="s">
+        <v>300</v>
+      </c>
+      <c r="E29" s="41" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A30" s="45">
+        <v>26</v>
+      </c>
+      <c r="B30" s="46" t="s">
+        <v>198</v>
+      </c>
+      <c r="C30" s="46" t="s">
+        <v>199</v>
+      </c>
+      <c r="D30" s="44" t="s">
+        <v>253</v>
+      </c>
+      <c r="E30" s="44" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A31" s="42">
+        <v>27</v>
+      </c>
+      <c r="B31" s="43" t="s">
+        <v>198</v>
+      </c>
+      <c r="C31" s="43" t="s">
         <v>214</v>
       </c>
-      <c r="C11" s="49" t="s">
-        <v>215</v>
-      </c>
-      <c r="D11" s="48" t="s">
-        <v>216</v>
-      </c>
-      <c r="E11" s="48" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A12" s="46">
-        <v>8</v>
-      </c>
-      <c r="B12" s="47" t="s">
+      <c r="D31" s="41" t="s">
+        <v>255</v>
+      </c>
+      <c r="E31" s="41" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" s="45">
+        <v>28</v>
+      </c>
+      <c r="B32" s="46" t="s">
+        <v>213</v>
+      </c>
+      <c r="C32" s="46" t="s">
         <v>199</v>
       </c>
-      <c r="C12" s="47" t="s">
-        <v>215</v>
-      </c>
-      <c r="D12" s="45" t="s">
-        <v>218</v>
-      </c>
-      <c r="E12" s="45" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="60" x14ac:dyDescent="0.25">
-      <c r="A13" s="50">
-        <v>9</v>
-      </c>
-      <c r="B13" s="49" t="s">
-        <v>214</v>
-      </c>
-      <c r="C13" s="49" t="s">
-        <v>203</v>
-      </c>
-      <c r="D13" s="48" t="s">
-        <v>220</v>
-      </c>
-      <c r="E13" s="48" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="46">
-        <v>10</v>
-      </c>
-      <c r="B14" s="47" t="s">
+      <c r="D32" s="44" t="s">
+        <v>257</v>
+      </c>
+      <c r="E32" s="44" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" s="42">
+        <v>29</v>
+      </c>
+      <c r="B33" s="43" t="s">
+        <v>198</v>
+      </c>
+      <c r="C33" s="43" t="s">
         <v>199</v>
       </c>
-      <c r="C14" s="47" t="s">
-        <v>203</v>
-      </c>
-      <c r="D14" s="45" t="s">
-        <v>222</v>
-      </c>
-      <c r="E14" s="45" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A15" s="43">
-        <v>11</v>
-      </c>
-      <c r="B15" s="44" t="s">
+      <c r="D33" s="41" t="s">
+        <v>259</v>
+      </c>
+      <c r="E33" s="41" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A34" s="45">
+        <v>30</v>
+      </c>
+      <c r="B34" s="46" t="s">
+        <v>198</v>
+      </c>
+      <c r="C34" s="46" t="s">
+        <v>202</v>
+      </c>
+      <c r="D34" s="44" t="s">
+        <v>261</v>
+      </c>
+      <c r="E34" s="44" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A35" s="42">
+        <v>31</v>
+      </c>
+      <c r="B35" s="43" t="s">
+        <v>198</v>
+      </c>
+      <c r="C35" s="43" t="s">
+        <v>202</v>
+      </c>
+      <c r="D35" s="41" t="s">
+        <v>263</v>
+      </c>
+      <c r="E35" s="41" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A36" s="45">
+        <v>32</v>
+      </c>
+      <c r="B36" s="46" t="s">
+        <v>198</v>
+      </c>
+      <c r="C36" s="46" t="s">
+        <v>202</v>
+      </c>
+      <c r="D36" s="44" t="s">
+        <v>265</v>
+      </c>
+      <c r="E36" s="44" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A37" s="42">
+        <v>33</v>
+      </c>
+      <c r="B37" s="43" t="s">
+        <v>198</v>
+      </c>
+      <c r="C37" s="43" t="s">
+        <v>202</v>
+      </c>
+      <c r="D37" s="41" t="s">
+        <v>267</v>
+      </c>
+      <c r="E37" s="41" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A38" s="45">
+        <v>34</v>
+      </c>
+      <c r="B38" s="46" t="s">
+        <v>198</v>
+      </c>
+      <c r="C38" s="46" t="s">
         <v>199</v>
       </c>
-      <c r="C15" s="44" t="s">
-        <v>215</v>
-      </c>
-      <c r="D15" s="42" t="s">
-        <v>224</v>
-      </c>
-      <c r="E15" s="42" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="46">
-        <v>12</v>
-      </c>
-      <c r="B16" s="47" t="s">
-        <v>214</v>
-      </c>
-      <c r="C16" s="47" t="s">
-        <v>200</v>
-      </c>
-      <c r="D16" s="45" t="s">
-        <v>226</v>
-      </c>
-      <c r="E16" s="45" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="50">
-        <v>13</v>
-      </c>
-      <c r="B17" s="49" t="s">
-        <v>214</v>
-      </c>
-      <c r="C17" s="49" t="s">
-        <v>228</v>
-      </c>
-      <c r="D17" s="48" t="s">
-        <v>229</v>
-      </c>
-      <c r="E17" s="48" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" s="46">
-        <v>14</v>
-      </c>
-      <c r="B18" s="47" t="s">
-        <v>199</v>
-      </c>
-      <c r="C18" s="47" t="s">
-        <v>215</v>
-      </c>
-      <c r="D18" s="45" t="s">
-        <v>231</v>
-      </c>
-      <c r="E18" s="45" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A19" s="43">
-        <v>15</v>
-      </c>
-      <c r="B19" s="44" t="s">
-        <v>199</v>
-      </c>
-      <c r="C19" s="44" t="s">
-        <v>200</v>
-      </c>
-      <c r="D19" s="42" t="s">
-        <v>233</v>
-      </c>
-      <c r="E19" s="42" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="46">
-        <v>16</v>
-      </c>
-      <c r="B20" s="47" t="s">
-        <v>199</v>
-      </c>
-      <c r="C20" s="47" t="s">
-        <v>200</v>
-      </c>
-      <c r="D20" s="45" t="s">
-        <v>235</v>
-      </c>
-      <c r="E20" s="45" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A21" s="43">
-        <v>17</v>
-      </c>
-      <c r="B21" s="44" t="s">
-        <v>199</v>
-      </c>
-      <c r="C21" s="44" t="s">
-        <v>215</v>
-      </c>
-      <c r="D21" s="42" t="s">
-        <v>237</v>
-      </c>
-      <c r="E21" s="42" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="46">
-        <v>18</v>
-      </c>
-      <c r="B22" s="47" t="s">
-        <v>214</v>
-      </c>
-      <c r="C22" s="47" t="s">
-        <v>228</v>
-      </c>
-      <c r="D22" s="45" t="s">
-        <v>239</v>
-      </c>
-      <c r="E22" s="45" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A23" s="43">
-        <v>19</v>
-      </c>
-      <c r="B23" s="44" t="s">
-        <v>214</v>
-      </c>
-      <c r="C23" s="44" t="s">
-        <v>200</v>
-      </c>
-      <c r="D23" s="42" t="s">
-        <v>241</v>
-      </c>
-      <c r="E23" s="42" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="46">
-        <v>20</v>
-      </c>
-      <c r="B24" s="47" t="s">
-        <v>199</v>
-      </c>
-      <c r="C24" s="47" t="s">
-        <v>203</v>
-      </c>
-      <c r="D24" s="45" t="s">
-        <v>243</v>
-      </c>
-      <c r="E24" s="45" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A25" s="43">
-        <v>21</v>
-      </c>
-      <c r="B25" s="44" t="s">
-        <v>199</v>
-      </c>
-      <c r="C25" s="44" t="s">
-        <v>203</v>
-      </c>
-      <c r="D25" s="42" t="s">
-        <v>245</v>
-      </c>
-      <c r="E25" s="42" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A26" s="46">
-        <v>22</v>
-      </c>
-      <c r="B26" s="47" t="s">
-        <v>247</v>
-      </c>
-      <c r="C26" s="47" t="s">
-        <v>200</v>
-      </c>
-      <c r="D26" s="45" t="s">
-        <v>248</v>
-      </c>
-      <c r="E26" s="45" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A27" s="43">
-        <v>23</v>
-      </c>
-      <c r="B27" s="44" t="s">
-        <v>199</v>
-      </c>
-      <c r="C27" s="44" t="s">
-        <v>203</v>
-      </c>
-      <c r="D27" s="42" t="s">
-        <v>250</v>
-      </c>
-      <c r="E27" s="42" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A28" s="46">
-        <v>24</v>
-      </c>
-      <c r="B28" s="47" t="s">
-        <v>199</v>
-      </c>
-      <c r="C28" s="47" t="s">
-        <v>203</v>
-      </c>
-      <c r="D28" s="45" t="s">
-        <v>252</v>
-      </c>
-      <c r="E28" s="45" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A29" s="43">
-        <v>25</v>
-      </c>
-      <c r="B29" s="44" t="s">
-        <v>199</v>
-      </c>
-      <c r="C29" s="44" t="s">
-        <v>203</v>
-      </c>
-      <c r="D29" s="42" t="s">
-        <v>254</v>
-      </c>
-      <c r="E29" s="42" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A30" s="46">
-        <v>26</v>
-      </c>
-      <c r="B30" s="47" t="s">
-        <v>199</v>
-      </c>
-      <c r="C30" s="47" t="s">
-        <v>200</v>
-      </c>
-      <c r="D30" s="45" t="s">
-        <v>256</v>
-      </c>
-      <c r="E30" s="45" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A31" s="43">
-        <v>27</v>
-      </c>
-      <c r="B31" s="44" t="s">
-        <v>199</v>
-      </c>
-      <c r="C31" s="44" t="s">
-        <v>215</v>
-      </c>
-      <c r="D31" s="42" t="s">
-        <v>258</v>
-      </c>
-      <c r="E31" s="42" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="46">
-        <v>28</v>
-      </c>
-      <c r="B32" s="47" t="s">
-        <v>214</v>
-      </c>
-      <c r="C32" s="47" t="s">
-        <v>200</v>
-      </c>
-      <c r="D32" s="45" t="s">
-        <v>260</v>
-      </c>
-      <c r="E32" s="45" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="43">
-        <v>29</v>
-      </c>
-      <c r="B33" s="44" t="s">
-        <v>199</v>
-      </c>
-      <c r="C33" s="44" t="s">
-        <v>200</v>
-      </c>
-      <c r="D33" s="42" t="s">
-        <v>262</v>
-      </c>
-      <c r="E33" s="42" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A34" s="46">
-        <v>30</v>
-      </c>
-      <c r="B34" s="47" t="s">
-        <v>199</v>
-      </c>
-      <c r="C34" s="47" t="s">
-        <v>203</v>
-      </c>
-      <c r="D34" s="45" t="s">
-        <v>264</v>
-      </c>
-      <c r="E34" s="45" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A35" s="43">
-        <v>31</v>
-      </c>
-      <c r="B35" s="44" t="s">
-        <v>199</v>
-      </c>
-      <c r="C35" s="44" t="s">
-        <v>203</v>
-      </c>
-      <c r="D35" s="42" t="s">
-        <v>266</v>
-      </c>
-      <c r="E35" s="42" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A36" s="46">
-        <v>32</v>
-      </c>
-      <c r="B36" s="47" t="s">
-        <v>199</v>
-      </c>
-      <c r="C36" s="47" t="s">
-        <v>203</v>
-      </c>
-      <c r="D36" s="45" t="s">
-        <v>268</v>
-      </c>
-      <c r="E36" s="45" t="s">
+      <c r="D38" s="44" t="s">
         <v>269</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A37" s="43">
-        <v>33</v>
-      </c>
-      <c r="B37" s="44" t="s">
-        <v>199</v>
-      </c>
-      <c r="C37" s="44" t="s">
-        <v>203</v>
-      </c>
-      <c r="D37" s="42" t="s">
+      <c r="E38" s="44" t="s">
         <v>270</v>
       </c>
-      <c r="E37" s="42" t="s">
+    </row>
+    <row r="39" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A39" s="42">
+        <v>35</v>
+      </c>
+      <c r="B39" s="43" t="s">
+        <v>198</v>
+      </c>
+      <c r="C39" s="43" t="s">
+        <v>202</v>
+      </c>
+      <c r="D39" s="41" t="s">
         <v>271</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A38" s="46">
-        <v>34</v>
-      </c>
-      <c r="B38" s="47" t="s">
-        <v>199</v>
-      </c>
-      <c r="C38" s="47" t="s">
-        <v>200</v>
-      </c>
-      <c r="D38" s="45" t="s">
+      <c r="E39" s="41" t="s">
         <v>272</v>
-      </c>
-      <c r="E38" s="45" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A39" s="43">
-        <v>35</v>
-      </c>
-      <c r="B39" s="44" t="s">
-        <v>199</v>
-      </c>
-      <c r="C39" s="44" t="s">
-        <v>203</v>
-      </c>
-      <c r="D39" s="42" t="s">
-        <v>274</v>
-      </c>
-      <c r="E39" s="42" t="s">
-        <v>275</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="53" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="B41" s="54"/>
       <c r="C41" s="54"/>
@@ -3185,11 +3420,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="65" t="s">
-        <v>151</v>
-      </c>
-      <c r="B1" s="65"/>
-      <c r="C1" s="65"/>
+      <c r="A1" s="66" t="s">
+        <v>150</v>
+      </c>
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
     </row>
     <row r="2" spans="1:3" ht="7.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
@@ -3198,202 +3433,193 @@
     </row>
     <row r="3" spans="1:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>152</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>153</v>
       </c>
       <c r="C3" s="3"/>
     </row>
     <row r="4" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="B4" s="69" t="s">
         <v>154</v>
       </c>
-      <c r="B4" s="67" t="s">
-        <v>155</v>
-      </c>
-      <c r="C4" s="68"/>
+      <c r="C4" s="70"/>
     </row>
     <row r="5" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="B5" s="68" t="s">
         <v>156</v>
       </c>
-      <c r="B5" s="69" t="s">
-        <v>157</v>
-      </c>
-      <c r="C5" s="60"/>
+      <c r="C5" s="56"/>
     </row>
     <row r="6" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="B6" s="69" t="s">
         <v>158</v>
       </c>
-      <c r="B6" s="67" t="s">
-        <v>159</v>
-      </c>
-      <c r="C6" s="60"/>
+      <c r="C6" s="56"/>
     </row>
     <row r="7" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="B7" s="68" t="s">
         <v>160</v>
       </c>
-      <c r="B7" s="69" t="s">
-        <v>161</v>
-      </c>
-      <c r="C7" s="60"/>
+      <c r="C7" s="56"/>
     </row>
     <row r="8" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="B8" s="69" t="s">
         <v>162</v>
       </c>
-      <c r="B8" s="67" t="s">
-        <v>163</v>
-      </c>
-      <c r="C8" s="60"/>
+      <c r="C8" s="56"/>
     </row>
     <row r="9" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="B9" s="68" t="s">
         <v>164</v>
       </c>
-      <c r="B9" s="69" t="s">
-        <v>165</v>
-      </c>
-      <c r="C9" s="60"/>
+      <c r="C9" s="56"/>
     </row>
     <row r="10" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="B10" s="69" t="s">
         <v>166</v>
       </c>
-      <c r="B10" s="67" t="s">
-        <v>167</v>
-      </c>
-      <c r="C10" s="60"/>
+      <c r="C10" s="56"/>
     </row>
     <row r="11" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="B11" s="68" t="s">
         <v>168</v>
       </c>
-      <c r="B11" s="69" t="s">
-        <v>169</v>
-      </c>
-      <c r="C11" s="60"/>
+      <c r="C11" s="56"/>
     </row>
     <row r="12" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="B12" s="69" t="s">
         <v>170</v>
       </c>
-      <c r="B12" s="67" t="s">
-        <v>171</v>
-      </c>
-      <c r="C12" s="60"/>
+      <c r="C12" s="56"/>
     </row>
     <row r="13" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="B13" s="68" t="s">
         <v>172</v>
       </c>
-      <c r="B13" s="69" t="s">
+      <c r="C13" s="56"/>
+    </row>
+    <row r="16" spans="1:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="59" t="s">
         <v>173</v>
       </c>
-      <c r="C13" s="60"/>
-    </row>
-    <row r="16" spans="1:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="61" t="s">
-        <v>174</v>
-      </c>
-      <c r="B16" s="61"/>
-      <c r="C16" s="61"/>
+      <c r="B16" s="59"/>
+      <c r="C16" s="59"/>
     </row>
     <row r="17" spans="1:3" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>175</v>
-      </c>
-      <c r="B17" s="62" t="s">
-        <v>25</v>
-      </c>
-      <c r="C17" s="63"/>
+        <v>174</v>
+      </c>
+      <c r="B17" s="60" t="s">
+        <v>24</v>
+      </c>
+      <c r="C17" s="61"/>
     </row>
     <row r="18" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B18" s="69" t="s">
         <v>176</v>
       </c>
-      <c r="B18" s="67" t="s">
-        <v>177</v>
-      </c>
-      <c r="C18" s="60"/>
+      <c r="C18" s="56"/>
     </row>
     <row r="19" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="B19" s="68" t="s">
         <v>178</v>
       </c>
-      <c r="B19" s="69" t="s">
-        <v>179</v>
-      </c>
-      <c r="C19" s="60"/>
+      <c r="C19" s="56"/>
     </row>
     <row r="20" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="B20" s="69" t="s">
         <v>180</v>
       </c>
-      <c r="B20" s="67" t="s">
-        <v>181</v>
-      </c>
-      <c r="C20" s="60"/>
+      <c r="C20" s="56"/>
     </row>
     <row r="21" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="B21" s="68" t="s">
         <v>182</v>
       </c>
-      <c r="B21" s="69" t="s">
-        <v>183</v>
-      </c>
-      <c r="C21" s="60"/>
+      <c r="C21" s="56"/>
     </row>
     <row r="22" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="B22" s="69" t="s">
         <v>184</v>
       </c>
-      <c r="B22" s="67" t="s">
-        <v>185</v>
-      </c>
-      <c r="C22" s="60"/>
+      <c r="C22" s="56"/>
     </row>
     <row r="23" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="B23" s="68" t="s">
         <v>186</v>
       </c>
-      <c r="B23" s="69" t="s">
-        <v>187</v>
-      </c>
-      <c r="C23" s="60"/>
+      <c r="C23" s="56"/>
     </row>
     <row r="24" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="B24" s="69" t="s">
         <v>188</v>
       </c>
-      <c r="B24" s="67" t="s">
-        <v>189</v>
-      </c>
-      <c r="C24" s="60"/>
+      <c r="C24" s="56"/>
     </row>
     <row r="25" spans="1:3" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="B25" s="68" t="s">
         <v>190</v>
       </c>
-      <c r="B25" s="69" t="s">
-        <v>191</v>
-      </c>
-      <c r="C25" s="60"/>
+      <c r="C25" s="56"/>
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
     <mergeCell ref="A16:C16"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="B4:C4"/>
@@ -3406,6 +3632,15 @@
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>